<commit_message>
update recommendation rules, tags and tried-perfume badge
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/perfumes-draft.xlsx
+++ b/docs/perfumes-draft.xlsx
@@ -1039,7 +1039,7 @@
       </c>
       <c r="M2" s="5" t="inlineStr">
         <is>
-          <t>clean, fresh, calm, cool, zesty</t>
+          <t>clean, fresh, zesty, cool, calm</t>
         </is>
       </c>
       <c r="N2" s="5" t="n"/>
@@ -1172,7 +1172,7 @@
       </c>
       <c r="M3" s="5" t="inlineStr">
         <is>
-          <t>clean, zesty, elegant, cool, fresh</t>
+          <t>fresh, zesty, clean, elegant, cool</t>
         </is>
       </c>
       <c r="N3" s="5" t="n"/>
@@ -1551,7 +1551,7 @@
       </c>
       <c r="M6" s="5" t="inlineStr">
         <is>
-          <t>soft, elegant, fresh, lovely, zesty, sweet</t>
+          <t>soft, fresh, elegant, lovely, sweet</t>
         </is>
       </c>
       <c r="N6" s="5" t="n"/>
@@ -1676,7 +1676,7 @@
       </c>
       <c r="M7" s="5" t="inlineStr">
         <is>
-          <t>soft, sweet, elegant, lovely, fresh, zesty</t>
+          <t>soft, lovely, fresh, sweet, elegant</t>
         </is>
       </c>
       <c r="N7" s="5" t="n"/>
@@ -1801,7 +1801,7 @@
       </c>
       <c r="M8" s="5" t="inlineStr">
         <is>
-          <t>sweet, cozy, warm, lovely, fresh, zesty</t>
+          <t>sweet, lovely, fresh, warm</t>
         </is>
       </c>
       <c r="N8" s="5" t="inlineStr">
@@ -1950,7 +1950,7 @@
       </c>
       <c r="M9" s="5" t="inlineStr">
         <is>
-          <t>soft, sweet, zesty, lovely, fresh</t>
+          <t>lovely, fresh, sweet, soft</t>
         </is>
       </c>
       <c r="N9" s="5" t="n"/>
@@ -2075,7 +2075,7 @@
       </c>
       <c r="M10" s="5" t="inlineStr">
         <is>
-          <t>elegant, warm, sweet, fresh, zesty, lovely</t>
+          <t>elegant, sweet, warm, lovely</t>
         </is>
       </c>
       <c r="N10" s="5" t="n"/>
@@ -2200,7 +2200,7 @@
       </c>
       <c r="M11" s="5" t="inlineStr">
         <is>
-          <t>cool, clean, fresh</t>
+          <t>cool, fresh, clean</t>
         </is>
       </c>
       <c r="N11" s="5" t="n"/>
@@ -2575,7 +2575,7 @@
       </c>
       <c r="M14" s="5" t="inlineStr">
         <is>
-          <t>fresh, calm, soft, cool</t>
+          <t>fresh, calm, soft</t>
         </is>
       </c>
       <c r="N14" s="5" t="n"/>
@@ -2825,7 +2825,7 @@
       </c>
       <c r="M16" s="5" t="inlineStr">
         <is>
-          <t>fresh, clean, calm, cool</t>
+          <t>clean, fresh, calm, cool</t>
         </is>
       </c>
       <c r="N16" s="5" t="n"/>
@@ -2950,7 +2950,7 @@
       </c>
       <c r="M17" s="5" t="inlineStr">
         <is>
-          <t>cool, deep, fresh, calm</t>
+          <t>fresh, deep, warm</t>
         </is>
       </c>
       <c r="N17" s="5" t="inlineStr">
@@ -2965,7 +2965,7 @@
       </c>
       <c r="P17" s="5" t="inlineStr">
         <is>
-          <t>mid</t>
+          <t>high</t>
         </is>
       </c>
       <c r="Q17" s="5" t="inlineStr">
@@ -3079,7 +3079,7 @@
       </c>
       <c r="M18" s="5" t="inlineStr">
         <is>
-          <t>calm, deep, clean</t>
+          <t>fresh, elegant, calm, deep</t>
         </is>
       </c>
       <c r="N18" s="5" t="n"/>
@@ -3204,7 +3204,7 @@
       </c>
       <c r="M19" s="5" t="inlineStr">
         <is>
-          <t>cozy, warm, sweet, calm</t>
+          <t>sweet, warm, sensual, cozy</t>
         </is>
       </c>
       <c r="N19" s="5" t="inlineStr">
@@ -3333,12 +3333,12 @@
       </c>
       <c r="M20" s="5" t="inlineStr">
         <is>
-          <t>elegant, sweet, warm, lovely</t>
+          <t>sweet, lovely, elegant, warm</t>
         </is>
       </c>
       <c r="N20" s="5" t="inlineStr">
         <is>
-          <t>heavyFloral, tooSweet, tooStrong, headache</t>
+          <t>heavyFloral, tooSweet, headache</t>
         </is>
       </c>
       <c r="O20" s="5" t="inlineStr">
@@ -3462,7 +3462,7 @@
       </c>
       <c r="M21" s="5" t="inlineStr">
         <is>
-          <t>elegant, soft, fresh, lovely</t>
+          <t>soft, lovely, fresh, elegant</t>
         </is>
       </c>
       <c r="N21" s="5" t="n"/>
@@ -3587,7 +3587,7 @@
       </c>
       <c r="M22" s="5" t="inlineStr">
         <is>
-          <t>elegant, soft, warm, lovely</t>
+          <t>soft, lovely, elegant, warm</t>
         </is>
       </c>
       <c r="N22" s="5" t="n"/>
@@ -3712,7 +3712,7 @@
       </c>
       <c r="M23" s="5" t="inlineStr">
         <is>
-          <t>elegant, warm, fresh, lovely</t>
+          <t>elegant, warm, lovely, fresh</t>
         </is>
       </c>
       <c r="N23" s="5" t="n"/>
@@ -3837,7 +3837,7 @@
       </c>
       <c r="M24" s="5" t="inlineStr">
         <is>
-          <t>elegant, sweet, soft, lovely, clean</t>
+          <t>elegant, lovely, sweet, soft</t>
         </is>
       </c>
       <c r="N24" s="5" t="n"/>
@@ -3962,7 +3962,7 @@
       </c>
       <c r="M25" s="5" t="inlineStr">
         <is>
-          <t>elegant, soft, lovely, clean</t>
+          <t>lovely, soft, elegant</t>
         </is>
       </c>
       <c r="N25" s="5" t="inlineStr">
@@ -4091,7 +4091,7 @@
       </c>
       <c r="M26" s="5" t="inlineStr">
         <is>
-          <t>elegant, soft, calm, clean, lovely</t>
+          <t>elegant, soft, calm, clean</t>
         </is>
       </c>
       <c r="N26" s="5" t="inlineStr">
@@ -4220,7 +4220,7 @@
       </c>
       <c r="M27" s="5" t="inlineStr">
         <is>
-          <t>elegant, calm, clean, lovely</t>
+          <t>elegant, clean, soft, calm</t>
         </is>
       </c>
       <c r="N27" s="5" t="inlineStr">
@@ -4349,7 +4349,7 @@
       </c>
       <c r="M28" s="5" t="inlineStr">
         <is>
-          <t>calm, soft, elegant, cozy, lovely</t>
+          <t>calm, soft, clean, elegant</t>
         </is>
       </c>
       <c r="N28" s="5" t="inlineStr">
@@ -4478,7 +4478,7 @@
       </c>
       <c r="M29" s="5" t="inlineStr">
         <is>
-          <t>calm, deep, soft, cozy, elegant</t>
+          <t>soft, elegant, cozy, deep, calm</t>
         </is>
       </c>
       <c r="N29" s="5" t="inlineStr">
@@ -4607,7 +4607,7 @@
       </c>
       <c r="M30" s="5" t="inlineStr">
         <is>
-          <t>soft, elegant, calm, lovely, cozy</t>
+          <t>soft, elegant, lovely, clean, calm</t>
         </is>
       </c>
       <c r="N30" s="5" t="inlineStr">
@@ -4736,7 +4736,7 @@
       </c>
       <c r="M31" s="5" t="inlineStr">
         <is>
-          <t>clean, soft, calm, cozy</t>
+          <t>clean, soft, calm</t>
         </is>
       </c>
       <c r="N31" s="5" t="inlineStr">
@@ -5034,14 +5034,10 @@
       </c>
       <c r="M33" s="5" t="inlineStr">
         <is>
-          <t>soft, elegant, warm, calm, clean, cozy</t>
-        </is>
-      </c>
-      <c r="N33" s="5" t="inlineStr">
-        <is>
-          <t>soapy</t>
-        </is>
-      </c>
+          <t>sensual, warm, elegant, cozy</t>
+        </is>
+      </c>
+      <c r="N33" s="5" t="n"/>
       <c r="O33" s="5" t="inlineStr">
         <is>
           <t>medium</t>
@@ -5163,7 +5159,7 @@
       </c>
       <c r="M34" s="5" t="inlineStr">
         <is>
-          <t>soft, clean, calm, cozy</t>
+          <t>soft, clean, cozy, calm</t>
         </is>
       </c>
       <c r="N34" s="5" t="inlineStr">
@@ -5292,7 +5288,7 @@
       </c>
       <c r="M35" s="5" t="inlineStr">
         <is>
-          <t>fresh, warm, sweet, calm, clean, cozy, soft</t>
+          <t>fresh, clean, warm, sweet, soft</t>
         </is>
       </c>
       <c r="N35" s="5" t="n"/>
@@ -5417,7 +5413,7 @@
       </c>
       <c r="M36" s="5" t="inlineStr">
         <is>
-          <t>deep, calm, warm, sensual</t>
+          <t>deep, warm, calm, fresh</t>
         </is>
       </c>
       <c r="N36" s="5" t="inlineStr">
@@ -5546,7 +5542,7 @@
       </c>
       <c r="M37" s="5" t="inlineStr">
         <is>
-          <t>warm, elegant, fresh</t>
+          <t>fresh, elegant, warm, lovely</t>
         </is>
       </c>
       <c r="N37" s="5" t="inlineStr">
@@ -5675,12 +5671,12 @@
       </c>
       <c r="M38" s="5" t="inlineStr">
         <is>
-          <t>deep, calm, warm, sensual</t>
+          <t>warm, deep, calm, cozy</t>
         </is>
       </c>
       <c r="N38" s="5" t="inlineStr">
         <is>
-          <t>tooStrong, smoky</t>
+          <t>smoky</t>
         </is>
       </c>
       <c r="O38" s="5" t="inlineStr">
@@ -5824,7 +5820,7 @@
       </c>
       <c r="M39" s="5" t="inlineStr">
         <is>
-          <t>calm, cozy, deep, warm</t>
+          <t>calm, warm, cozy, elegant</t>
         </is>
       </c>
       <c r="N39" s="5" t="n"/>
@@ -5949,12 +5945,12 @@
       </c>
       <c r="M40" s="5" t="inlineStr">
         <is>
-          <t>deep, warm, elegant, sensual, calm</t>
+          <t>elegant, deep, warm, sensual</t>
         </is>
       </c>
       <c r="N40" s="5" t="inlineStr">
         <is>
-          <t>tooStrong, smoky, spicy</t>
+          <t>smoky</t>
         </is>
       </c>
       <c r="O40" s="5" t="inlineStr">
@@ -6078,7 +6074,7 @@
       </c>
       <c r="M41" s="5" t="inlineStr">
         <is>
-          <t>calm, cozy, soft, warm, deep</t>
+          <t>calm, fresh, warm, cozy</t>
         </is>
       </c>
       <c r="N41" s="5" t="n"/>
@@ -6223,12 +6219,12 @@
       </c>
       <c r="M42" s="5" t="inlineStr">
         <is>
-          <t>warm, elegant, sweet, sensual, cozy, deep</t>
+          <t>sweet, warm, elegant, cozy</t>
         </is>
       </c>
       <c r="N42" s="5" t="inlineStr">
         <is>
-          <t>tooSweet, tooStrong</t>
+          <t>tooSweet</t>
         </is>
       </c>
       <c r="O42" s="5" t="inlineStr">
@@ -6352,12 +6348,12 @@
       </c>
       <c r="M43" s="5" t="inlineStr">
         <is>
-          <t>warm, deep, elegant, sensual, cozy, sweet</t>
+          <t>warm, sensual, elegant, deep, sweet</t>
         </is>
       </c>
       <c r="N43" s="5" t="inlineStr">
         <is>
-          <t>tooStrong, powdery</t>
+          <t>powdery</t>
         </is>
       </c>
       <c r="O43" s="5" t="inlineStr">
@@ -6481,7 +6477,7 @@
       </c>
       <c r="M44" s="5" t="inlineStr">
         <is>
-          <t>warm, elegant, soft, cozy, sweet, deep</t>
+          <t>warm, elegant, soft, sweet</t>
         </is>
       </c>
       <c r="N44" s="5" t="n"/>
@@ -6606,12 +6602,12 @@
       </c>
       <c r="M45" s="5" t="inlineStr">
         <is>
-          <t>sweet, deep, warm, sensual, cozy</t>
+          <t>sweet, sensual, warm, deep</t>
         </is>
       </c>
       <c r="N45" s="5" t="inlineStr">
         <is>
-          <t>tooSweet, tooStrong</t>
+          <t>tooSweet</t>
         </is>
       </c>
       <c r="O45" s="5" t="inlineStr">
@@ -6735,7 +6731,7 @@
       </c>
       <c r="M46" s="5" t="inlineStr">
         <is>
-          <t>sweet, cozy, elegant, lovely, warm</t>
+          <t>sweet, lovely, cozy, elegant</t>
         </is>
       </c>
       <c r="N46" s="5" t="inlineStr">
@@ -6864,12 +6860,12 @@
       </c>
       <c r="M47" s="5" t="inlineStr">
         <is>
-          <t>warm, cozy, deep, sensual, sweet</t>
+          <t>warm, sweet, cozy, sensual, deep</t>
         </is>
       </c>
       <c r="N47" s="5" t="inlineStr">
         <is>
-          <t>tooSweet, tooStrong</t>
+          <t>tooSweet</t>
         </is>
       </c>
       <c r="O47" s="5" t="inlineStr">
@@ -6993,12 +6989,12 @@
       </c>
       <c r="M48" s="5" t="inlineStr">
         <is>
-          <t>sweet, deep, warm, sensual, cozy</t>
+          <t>sweet, deep, sensual, warm</t>
         </is>
       </c>
       <c r="N48" s="5" t="inlineStr">
         <is>
-          <t>tooSweet, tooStrong, headache</t>
+          <t>tooSweet, headache</t>
         </is>
       </c>
       <c r="O48" s="5" t="inlineStr">
@@ -7122,7 +7118,7 @@
       </c>
       <c r="M49" s="5" t="inlineStr">
         <is>
-          <t>cozy, warm, deep, sensual</t>
+          <t>cozy, warm, deep, sweet</t>
         </is>
       </c>
       <c r="N49" s="5" t="inlineStr">
@@ -7271,7 +7267,7 @@
       </c>
       <c r="M50" s="5" t="inlineStr">
         <is>
-          <t>deep, cozy, warm, sensual</t>
+          <t>warm, cozy, deep, sensual</t>
         </is>
       </c>
       <c r="N50" s="5" t="inlineStr">
@@ -7400,12 +7396,12 @@
       </c>
       <c r="M51" s="5" t="inlineStr">
         <is>
-          <t>deep, warm, cozy, sensual</t>
+          <t>warm, cozy, deep, sweet, sensual</t>
         </is>
       </c>
       <c r="N51" s="5" t="inlineStr">
         <is>
-          <t>tooSweet, tooStrong, smoky, spicy</t>
+          <t>tooSweet, smoky</t>
         </is>
       </c>
       <c r="O51" s="5" t="inlineStr">
@@ -7529,7 +7525,7 @@
       </c>
       <c r="M52" s="5" t="inlineStr">
         <is>
-          <t>clean, soft, calm, cozy</t>
+          <t>clean, soft, calm</t>
         </is>
       </c>
       <c r="N52" s="5" t="n"/>
@@ -7540,7 +7536,7 @@
       </c>
       <c r="P52" s="5" t="inlineStr">
         <is>
-          <t>mid</t>
+          <t>high</t>
         </is>
       </c>
       <c r="Q52" s="5" t="inlineStr">
@@ -7674,12 +7670,12 @@
       </c>
       <c r="M53" s="5" t="inlineStr">
         <is>
-          <t>deep, warm, elegant, sensual</t>
+          <t>elegant, deep, warm, sensual</t>
         </is>
       </c>
       <c r="N53" s="5" t="inlineStr">
         <is>
-          <t>tooStrong, spicy, smoky</t>
+          <t>spicy, smoky</t>
         </is>
       </c>
       <c r="O53" s="5" t="inlineStr">
@@ -7823,7 +7819,7 @@
       </c>
       <c r="M54" s="5" t="inlineStr">
         <is>
-          <t>calm, cozy, deep, fresh</t>
+          <t>calm, cozy, deep</t>
         </is>
       </c>
       <c r="N54" s="5" t="inlineStr">
@@ -7972,7 +7968,7 @@
       </c>
       <c r="M55" s="5" t="inlineStr">
         <is>
-          <t>fresh, clean, zesty, cool</t>
+          <t>fresh, zesty, clean, cool</t>
         </is>
       </c>
       <c r="N55" s="5" t="n"/>
@@ -8117,12 +8113,12 @@
       </c>
       <c r="M56" s="5" t="inlineStr">
         <is>
-          <t>sweet, soft, elegant, cozy, warm</t>
+          <t>sweet, soft, cozy, warm, lovely</t>
         </is>
       </c>
       <c r="N56" s="5" t="inlineStr">
         <is>
-          <t>tooSweet, tooStrong</t>
+          <t>tooSweet</t>
         </is>
       </c>
       <c r="O56" s="5" t="inlineStr">
@@ -8246,12 +8242,12 @@
       </c>
       <c r="M57" s="5" t="inlineStr">
         <is>
-          <t>deep, sweet, warm, sensual, cozy</t>
+          <t>sweet, deep, warm, sensual, cozy</t>
         </is>
       </c>
       <c r="N57" s="5" t="inlineStr">
         <is>
-          <t>tooSweet, tooStrong</t>
+          <t>tooSweet</t>
         </is>
       </c>
       <c r="O57" s="5" t="inlineStr">
@@ -8375,12 +8371,12 @@
       </c>
       <c r="M58" s="5" t="inlineStr">
         <is>
-          <t>fresh, deep, elegant, sweet</t>
+          <t>fresh, elegant, sweet, deep</t>
         </is>
       </c>
       <c r="N58" s="5" t="inlineStr">
         <is>
-          <t>smoky, tooStrong</t>
+          <t>smoky</t>
         </is>
       </c>
       <c r="O58" s="5" t="inlineStr">
@@ -8504,7 +8500,7 @@
       </c>
       <c r="M59" s="5" t="inlineStr">
         <is>
-          <t>fresh, clean, cool</t>
+          <t>fresh, cool, clean</t>
         </is>
       </c>
       <c r="N59" s="5" t="n"/>
@@ -8754,7 +8750,7 @@
       </c>
       <c r="M61" s="5" t="inlineStr">
         <is>
-          <t>cool, fresh, clean</t>
+          <t>fresh, cool, clean, elegant</t>
         </is>
       </c>
       <c r="N61" s="5" t="n"/>
@@ -8884,7 +8880,7 @@
       </c>
       <c r="N62" s="5" t="inlineStr">
         <is>
-          <t>tooStrong, heavyFloral, spicy, smoky</t>
+          <t>heavyFloral, spicy, smoky</t>
         </is>
       </c>
       <c r="O62" s="5" t="inlineStr">
@@ -9008,12 +9004,12 @@
       </c>
       <c r="M63" s="5" t="inlineStr">
         <is>
-          <t>warm, cozy, deep, sensual, calm</t>
+          <t>warm, cozy, sensual, deep</t>
         </is>
       </c>
       <c r="N63" s="5" t="inlineStr">
         <is>
-          <t>tooStrong, spicy</t>
+          <t>spicy</t>
         </is>
       </c>
       <c r="O63" s="5" t="inlineStr">
@@ -9137,12 +9133,12 @@
       </c>
       <c r="M64" s="5" t="inlineStr">
         <is>
-          <t>elegant, warm, sensual</t>
+          <t>elegant, sensual, warm</t>
         </is>
       </c>
       <c r="N64" s="5" t="inlineStr">
         <is>
-          <t>heavyFloral, tooStrong, headache</t>
+          <t>heavyFloral, headache</t>
         </is>
       </c>
       <c r="O64" s="5" t="inlineStr">
@@ -9266,7 +9262,7 @@
       </c>
       <c r="M65" s="5" t="inlineStr">
         <is>
-          <t>fresh, soft, calm, cool</t>
+          <t>fresh, soft, cool, calm</t>
         </is>
       </c>
       <c r="N65" s="5" t="inlineStr">
@@ -9395,7 +9391,7 @@
       </c>
       <c r="M66" s="5" t="inlineStr">
         <is>
-          <t>soft, elegant, sweet, lovely, calm, cozy</t>
+          <t>soft, sweet, lovely, elegant</t>
         </is>
       </c>
       <c r="N66" s="5" t="inlineStr">
@@ -9649,7 +9645,7 @@
       </c>
       <c r="M68" s="5" t="inlineStr">
         <is>
-          <t>sweet, soft, fresh, lovely, zesty</t>
+          <t>lovely, sweet, soft, fresh</t>
         </is>
       </c>
       <c r="N68" s="5" t="n"/>
@@ -9774,7 +9770,7 @@
       </c>
       <c r="M69" s="5" t="inlineStr">
         <is>
-          <t>calm, deep, fresh, warm</t>
+          <t>calm, deep, fresh</t>
         </is>
       </c>
       <c r="N69" s="5" t="inlineStr">
@@ -9923,7 +9919,7 @@
       </c>
       <c r="M70" s="5" t="inlineStr">
         <is>
-          <t>fresh, clean, cool, zesty</t>
+          <t>fresh, zesty, clean, cool</t>
         </is>
       </c>
       <c r="N70" s="5" t="n"/>
@@ -10068,7 +10064,7 @@
       </c>
       <c r="M71" s="5" t="inlineStr">
         <is>
-          <t>elegant, sweet, soft, lovely</t>
+          <t>lovely, elegant, sweet, soft</t>
         </is>
       </c>
       <c r="N71" s="5" t="n"/>
@@ -10193,7 +10189,7 @@
       </c>
       <c r="M72" s="5" t="inlineStr">
         <is>
-          <t>warm, deep, elegant, calm</t>
+          <t>warm, elegant, sweet, deep</t>
         </is>
       </c>
       <c r="N72" s="5" t="inlineStr">
@@ -10451,14 +10447,10 @@
       </c>
       <c r="M74" s="5" t="inlineStr">
         <is>
-          <t>deep, elegant, warm, sensual, calm</t>
-        </is>
-      </c>
-      <c r="N74" s="5" t="inlineStr">
-        <is>
-          <t>tooStrong, smoky</t>
-        </is>
-      </c>
+          <t>sensual, deep, warm, elegant</t>
+        </is>
+      </c>
+      <c r="N74" s="5" t="n"/>
       <c r="O74" s="5" t="inlineStr">
         <is>
           <t>strong</t>
@@ -10466,7 +10458,7 @@
       </c>
       <c r="P74" s="5" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>mid</t>
         </is>
       </c>
       <c r="Q74" s="5" t="inlineStr">
@@ -10580,7 +10572,7 @@
       </c>
       <c r="M75" s="5" t="inlineStr">
         <is>
-          <t>warm, deep, cozy, sensual, sweet</t>
+          <t>warm, sensual, cozy, deep, sweet</t>
         </is>
       </c>
       <c r="N75" s="5" t="inlineStr">
@@ -10709,7 +10701,7 @@
       </c>
       <c r="M76" s="5" t="inlineStr">
         <is>
-          <t>warm, cozy, soft, sweet, deep</t>
+          <t>warm, soft, cozy, sweet</t>
         </is>
       </c>
       <c r="N76" s="5" t="n"/>
@@ -10834,7 +10826,7 @@
       </c>
       <c r="M77" s="5" t="inlineStr">
         <is>
-          <t>deep, warm, elegant, sensual, calm</t>
+          <t>deep, warm, sensual, elegant</t>
         </is>
       </c>
       <c r="N77" s="5" t="inlineStr">
@@ -10963,7 +10955,7 @@
       </c>
       <c r="M78" s="5" t="inlineStr">
         <is>
-          <t>fresh, zesty, elegant, sweet, lovely</t>
+          <t>fresh, zesty, elegant</t>
         </is>
       </c>
       <c r="N78" s="5" t="n"/>
@@ -11088,10 +11080,14 @@
       </c>
       <c r="M79" s="5" t="inlineStr">
         <is>
-          <t>soft, calm, clean, cozy</t>
-        </is>
-      </c>
-      <c r="N79" s="5" t="n"/>
+          <t>soft, clean, calm, lovely</t>
+        </is>
+      </c>
+      <c r="N79" s="5" t="inlineStr">
+        <is>
+          <t>powdery</t>
+        </is>
+      </c>
       <c r="O79" s="5" t="inlineStr">
         <is>
           <t>medium</t>
@@ -11233,7 +11229,7 @@
       </c>
       <c r="M80" s="5" t="inlineStr">
         <is>
-          <t>fresh, warm, soft, clean, zesty</t>
+          <t>fresh, zesty, soft, clean, warm</t>
         </is>
       </c>
       <c r="N80" s="5" t="n"/>
@@ -11523,7 +11519,7 @@
       </c>
       <c r="M82" s="5" t="inlineStr">
         <is>
-          <t>cozy, warm, soft, deep</t>
+          <t>cozy, warm, soft</t>
         </is>
       </c>
       <c r="N82" s="5" t="n"/>
@@ -11668,7 +11664,7 @@
       </c>
       <c r="M83" s="5" t="inlineStr">
         <is>
-          <t>warm, cozy, soft</t>
+          <t>warm, cozy, soft, calm</t>
         </is>
       </c>
       <c r="N83" s="5" t="inlineStr">
@@ -11797,7 +11793,7 @@
       </c>
       <c r="M84" s="5" t="inlineStr">
         <is>
-          <t>calm, cozy, elegant, warm, deep</t>
+          <t>warm, elegant, cozy, calm</t>
         </is>
       </c>
       <c r="N84" s="5" t="n"/>
@@ -11922,7 +11918,7 @@
       </c>
       <c r="M85" s="5" t="inlineStr">
         <is>
-          <t>sweet, warm, elegant, sensual, cozy</t>
+          <t>sweet, sensual, warm, elegant</t>
         </is>
       </c>
       <c r="N85" s="5" t="inlineStr">
@@ -12051,7 +12047,7 @@
       </c>
       <c r="M86" s="5" t="inlineStr">
         <is>
-          <t>warm, sweet, elegant, sensual</t>
+          <t>warm, sweet, elegant</t>
         </is>
       </c>
       <c r="N86" s="5" t="n"/>
@@ -12305,7 +12301,7 @@
       </c>
       <c r="M88" s="5" t="inlineStr">
         <is>
-          <t>deep, elegant, warm, sensual</t>
+          <t>sensual, deep, elegant, warm</t>
         </is>
       </c>
       <c r="N88" s="5" t="inlineStr">
@@ -12434,7 +12430,7 @@
       </c>
       <c r="M89" s="5" t="inlineStr">
         <is>
-          <t>deep, warm, sensual</t>
+          <t>warm, sensual, deep</t>
         </is>
       </c>
       <c r="N89" s="5" t="inlineStr">
@@ -12563,7 +12559,7 @@
       </c>
       <c r="M90" s="5" t="inlineStr">
         <is>
-          <t>calm, warm, fresh, deep</t>
+          <t>calm, fresh, warm, elegant</t>
         </is>
       </c>
       <c r="N90" s="5" t="n"/>
@@ -12688,7 +12684,7 @@
       </c>
       <c r="M91" s="5" t="inlineStr">
         <is>
-          <t>fresh, zesty, cool</t>
+          <t>fresh, zesty, cool, clean</t>
         </is>
       </c>
       <c r="N91" s="5" t="n"/>
@@ -12938,7 +12934,7 @@
       </c>
       <c r="M93" s="5" t="inlineStr">
         <is>
-          <t>zesty, fresh, warm, clean</t>
+          <t>zesty, fresh, sweet, clean</t>
         </is>
       </c>
       <c r="N93" s="5" t="n"/>
@@ -13063,7 +13059,7 @@
       </c>
       <c r="M94" s="5" t="inlineStr">
         <is>
-          <t>warm, sweet, deep, sensual, cozy</t>
+          <t>sweet, warm, cozy, sensual, deep</t>
         </is>
       </c>
       <c r="N94" s="5" t="inlineStr">
@@ -13184,7 +13180,7 @@
       </c>
       <c r="M95" s="5" t="inlineStr">
         <is>
-          <t>clean, soft, calm, warm</t>
+          <t>clean, soft, calm</t>
         </is>
       </c>
       <c r="N95" s="5" t="n"/>
@@ -13543,7 +13539,7 @@
       </c>
       <c r="M98" s="5" t="inlineStr">
         <is>
-          <t>sweet, elegant, soft, lovely</t>
+          <t>lovely, sweet, elegant, soft</t>
         </is>
       </c>
       <c r="N98" s="5" t="n"/>
@@ -13797,7 +13793,7 @@
       </c>
       <c r="M100" s="5" t="inlineStr">
         <is>
-          <t>warm, cozy, deep, sensual, sweet</t>
+          <t>warm, cozy, sweet, deep</t>
         </is>
       </c>
       <c r="N100" s="5" t="inlineStr">
@@ -13926,7 +13922,7 @@
       </c>
       <c r="M101" s="5" t="inlineStr">
         <is>
-          <t>lovely, fresh, soft, elegant</t>
+          <t>fresh, zesty, lovely, soft</t>
         </is>
       </c>
       <c r="N101" s="5" t="n"/>
@@ -14051,7 +14047,7 @@
       </c>
       <c r="M102" s="5" t="inlineStr">
         <is>
-          <t>fresh, sweet, warm, calm</t>
+          <t>fresh, sweet, warm</t>
         </is>
       </c>
       <c r="N102" s="5" t="inlineStr">
@@ -14180,7 +14176,7 @@
       </c>
       <c r="M103" s="5" t="inlineStr">
         <is>
-          <t>warm, deep, sensual, cozy, sweet</t>
+          <t>sweet, warm, sensual, deep</t>
         </is>
       </c>
       <c r="N103" s="5" t="inlineStr">
@@ -14309,7 +14305,7 @@
       </c>
       <c r="M104" s="5" t="inlineStr">
         <is>
-          <t>sweet, lovely, elegant, cozy, warm</t>
+          <t>sweet, lovely, elegant</t>
         </is>
       </c>
       <c r="N104" s="5" t="inlineStr">
@@ -14438,7 +14434,7 @@
       </c>
       <c r="M105" s="5" t="inlineStr">
         <is>
-          <t>calm, warm, fresh, deep</t>
+          <t>fresh, warm, calm</t>
         </is>
       </c>
       <c r="N105" s="5" t="inlineStr">
@@ -14567,7 +14563,7 @@
       </c>
       <c r="M106" s="5" t="inlineStr">
         <is>
-          <t>soft, elegant, clean, lovely</t>
+          <t>clean, soft, lovely, elegant</t>
         </is>
       </c>
       <c r="N106" s="5" t="n"/>
@@ -14692,7 +14688,7 @@
       </c>
       <c r="M107" s="5" t="inlineStr">
         <is>
-          <t>sweet, sensual, elegant, cozy, warm</t>
+          <t>sweet, sensual, elegant, warm</t>
         </is>
       </c>
       <c r="N107" s="5" t="inlineStr">
@@ -14821,7 +14817,7 @@
       </c>
       <c r="M108" s="5" t="inlineStr">
         <is>
-          <t>cool, fresh, deep, calm</t>
+          <t>fresh, cool, calm</t>
         </is>
       </c>
       <c r="N108" s="5" t="n"/>
@@ -15071,7 +15067,7 @@
       </c>
       <c r="M110" s="5" t="inlineStr">
         <is>
-          <t>calm, deep, fresh, warm</t>
+          <t>fresh, warm, deep</t>
         </is>
       </c>
       <c r="N110" s="5" t="n"/>
@@ -15446,7 +15442,7 @@
       </c>
       <c r="M113" s="5" t="inlineStr">
         <is>
-          <t>sweet, lovely, elegant, fresh, zesty</t>
+          <t>sweet, lovely, fresh, elegant</t>
         </is>
       </c>
       <c r="N113" s="5" t="inlineStr">
@@ -15580,7 +15576,7 @@
       </c>
       <c r="N114" s="5" t="inlineStr">
         <is>
-          <t>tooSweet</t>
+          <t>tooSweet, powdery</t>
         </is>
       </c>
       <c r="O114" s="5" t="inlineStr">
@@ -15704,12 +15700,12 @@
       </c>
       <c r="M115" s="5" t="inlineStr">
         <is>
-          <t>elegant, deep, sensual</t>
+          <t>sensual, deep, elegant, warm</t>
         </is>
       </c>
       <c r="N115" s="5" t="inlineStr">
         <is>
-          <t>heavyFloral, tooStrong, headache</t>
+          <t>heavyFloral, headache</t>
         </is>
       </c>
       <c r="O115" s="5" t="inlineStr">
@@ -16333,7 +16329,7 @@
       </c>
       <c r="M120" s="5" t="inlineStr">
         <is>
-          <t>elegant, soft, calm, cozy, lovely</t>
+          <t>elegant, soft, calm, cozy</t>
         </is>
       </c>
       <c r="N120" s="5" t="inlineStr">
@@ -16462,7 +16458,7 @@
       </c>
       <c r="M121" s="5" t="inlineStr">
         <is>
-          <t>sensual, warm, deep, cozy, sweet</t>
+          <t>sensual, sweet, warm, deep</t>
         </is>
       </c>
       <c r="N121" s="5" t="inlineStr">
@@ -17099,7 +17095,7 @@
       </c>
       <c r="M126" s="5" t="inlineStr">
         <is>
-          <t>warm, soft, elegant, cozy, sweet, deep</t>
+          <t>warm, soft, cozy, elegant</t>
         </is>
       </c>
       <c r="N126" s="5" t="n"/>
@@ -17389,7 +17385,7 @@
       </c>
       <c r="M128" s="5" t="inlineStr">
         <is>
-          <t>fresh, calm, clean, warm</t>
+          <t>fresh, clean, calm</t>
         </is>
       </c>
       <c r="N128" s="5" t="n"/>
@@ -17812,7 +17808,7 @@
       </c>
       <c r="M131" s="5" t="inlineStr">
         <is>
-          <t>elegant, warm, sensual, calm, deep</t>
+          <t>sensual, warm, elegant, deep</t>
         </is>
       </c>
       <c r="N131" s="5" t="n"/>
@@ -18191,7 +18187,7 @@
       </c>
       <c r="M134" s="5" t="inlineStr">
         <is>
-          <t>deep, warm, sensual, calm</t>
+          <t>deep, warm, sensual</t>
         </is>
       </c>
       <c r="N134" s="5" t="inlineStr">
@@ -18953,7 +18949,7 @@
       </c>
       <c r="M140" s="5" t="inlineStr">
         <is>
-          <t>clean, soft, elegant, calm, cozy, lovely</t>
+          <t>clean, soft, elegant, calm</t>
         </is>
       </c>
       <c r="N140" s="5" t="inlineStr">
@@ -19082,7 +19078,7 @@
       </c>
       <c r="M141" s="5" t="inlineStr">
         <is>
-          <t>lovely, soft, elegant</t>
+          <t>lovely, soft, elegant, warm</t>
         </is>
       </c>
       <c r="N141" s="5" t="inlineStr">
@@ -19211,7 +19207,7 @@
       </c>
       <c r="M142" s="5" t="inlineStr">
         <is>
-          <t>lovely, fresh, soft, clean, elegant</t>
+          <t>lovely, fresh, soft, elegant</t>
         </is>
       </c>
       <c r="N142" s="5" t="n"/>
@@ -19336,7 +19332,7 @@
       </c>
       <c r="M143" s="5" t="inlineStr">
         <is>
-          <t>calm, soft, clean, cool</t>
+          <t>calm, soft, cozy, clean</t>
         </is>
       </c>
       <c r="N143" s="5" t="n"/>
@@ -19755,7 +19751,7 @@
       </c>
       <c r="M146" s="5" t="inlineStr">
         <is>
-          <t>fresh, cool, calm</t>
+          <t>fresh, cool, clean</t>
         </is>
       </c>
       <c r="N146" s="5" t="n"/>
@@ -20005,7 +20001,7 @@
       </c>
       <c r="M148" s="5" t="inlineStr">
         <is>
-          <t>sensual, warm, sweet, cozy</t>
+          <t>sweet, sensual, warm</t>
         </is>
       </c>
       <c r="N148" s="5" t="inlineStr">
@@ -20134,7 +20130,7 @@
       </c>
       <c r="M149" s="5" t="inlineStr">
         <is>
-          <t>sweet, warm, sensual, cozy</t>
+          <t>sweet, warm, cozy, fresh</t>
         </is>
       </c>
       <c r="N149" s="5" t="inlineStr">
@@ -20388,7 +20384,7 @@
       </c>
       <c r="M151" s="5" t="inlineStr">
         <is>
-          <t>soft, lovely, fresh, elegant</t>
+          <t>soft, fresh, lovely, sweet</t>
         </is>
       </c>
       <c r="N151" s="5" t="n"/>
@@ -20638,10 +20634,14 @@
       </c>
       <c r="M153" s="5" t="inlineStr">
         <is>
-          <t>clean, calm, soft, lovely, elegant</t>
-        </is>
-      </c>
-      <c r="N153" s="5" t="n"/>
+          <t>clean, calm, soft, elegant</t>
+        </is>
+      </c>
+      <c r="N153" s="5" t="inlineStr">
+        <is>
+          <t>soapy</t>
+        </is>
+      </c>
       <c r="O153" s="5" t="inlineStr">
         <is>
           <t>light</t>
@@ -21021,7 +21021,7 @@
       </c>
       <c r="M156" s="5" t="inlineStr">
         <is>
-          <t>cool, fresh, clean, calm</t>
+          <t>fresh, cool, clean</t>
         </is>
       </c>
       <c r="N156" s="5" t="n"/>
@@ -21154,12 +21154,12 @@
       </c>
       <c r="M157" s="5" t="inlineStr">
         <is>
-          <t>warm, elegant, sensual</t>
+          <t>warm, sensual, elegant, sweet</t>
         </is>
       </c>
       <c r="N157" s="5" t="inlineStr">
         <is>
-          <t>heavyFloral</t>
+          <t>powdery</t>
         </is>
       </c>
       <c r="O157" s="5" t="inlineStr">
@@ -21283,7 +21283,7 @@
       </c>
       <c r="M158" s="5" t="inlineStr">
         <is>
-          <t>elegant, soft, calm, lovely</t>
+          <t>soft, fresh, elegant, calm</t>
         </is>
       </c>
       <c r="N158" s="5" t="n"/>
@@ -21665,7 +21665,11 @@
           <t>soft, clean, cozy, calm</t>
         </is>
       </c>
-      <c r="N161" s="5" t="n"/>
+      <c r="N161" s="5" t="inlineStr">
+        <is>
+          <t>powdery, soapy</t>
+        </is>
+      </c>
       <c r="O161" s="5" t="inlineStr">
         <is>
           <t>medium</t>
@@ -21791,7 +21795,7 @@
       </c>
       <c r="M162" s="5" t="inlineStr">
         <is>
-          <t>calm, soft, cozy, warm, deep</t>
+          <t>calm, soft, cozy, warm</t>
         </is>
       </c>
       <c r="N162" s="5" t="n"/>
@@ -22504,7 +22508,7 @@
       </c>
       <c r="M167" s="5" t="inlineStr">
         <is>
-          <t>fresh, lovely, soft, zesty, sweet</t>
+          <t>fresh, zesty, sweet, lovely</t>
         </is>
       </c>
       <c r="N167" s="5" t="n"/>
@@ -22629,7 +22633,7 @@
       </c>
       <c r="M168" s="5" t="inlineStr">
         <is>
-          <t>clean, calm, cool</t>
+          <t>clean, fresh, calm, cool</t>
         </is>
       </c>
       <c r="N168" s="5" t="n"/>
@@ -22754,7 +22758,7 @@
       </c>
       <c r="M169" s="5" t="inlineStr">
         <is>
-          <t>lovely, sweet, soft, fresh, zesty</t>
+          <t>lovely, sweet, soft, fresh</t>
         </is>
       </c>
       <c r="N169" s="5" t="n"/>
@@ -23540,7 +23544,7 @@
       </c>
       <c r="M175" s="5" t="inlineStr">
         <is>
-          <t>fresh, elegant, lovely</t>
+          <t>fresh, soft, lovely, elegant</t>
         </is>
       </c>
       <c r="N175" s="5" t="n"/>
@@ -23677,7 +23681,7 @@
       </c>
       <c r="M176" s="5" t="inlineStr">
         <is>
-          <t>calm, fresh, elegant, warm, deep</t>
+          <t>fresh, calm, elegant, deep</t>
         </is>
       </c>
       <c r="N176" s="5" t="n"/>
@@ -23951,7 +23955,7 @@
       </c>
       <c r="M178" s="5" t="inlineStr">
         <is>
-          <t>calm, deep, soft, warm</t>
+          <t>calm, soft, warm, elegant</t>
         </is>
       </c>
       <c r="N178" s="5" t="n"/>
@@ -24362,10 +24366,14 @@
       </c>
       <c r="M181" s="5" t="inlineStr">
         <is>
-          <t>zesty, lovely, soft, clean, cool, fresh</t>
-        </is>
-      </c>
-      <c r="N181" s="5" t="n"/>
+          <t>zesty, fresh, clean, sweet, soft</t>
+        </is>
+      </c>
+      <c r="N181" s="5" t="inlineStr">
+        <is>
+          <t>soapy</t>
+        </is>
+      </c>
       <c r="O181" s="5" t="inlineStr">
         <is>
           <t>light</t>
@@ -24373,7 +24381,7 @@
       </c>
       <c r="P181" s="5" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="Q181" s="5" t="inlineStr">
@@ -24495,7 +24503,7 @@
       </c>
       <c r="M182" s="5" t="inlineStr">
         <is>
-          <t>calm, fresh, soft, cool</t>
+          <t>calm, fresh, soft, cozy</t>
         </is>
       </c>
       <c r="N182" s="5" t="n"/>
@@ -24785,7 +24793,7 @@
       </c>
       <c r="M184" s="5" t="inlineStr">
         <is>
-          <t>elegant, soft, lovely, clean</t>
+          <t>elegant, soft, lovely, sweet</t>
         </is>
       </c>
       <c r="N184" s="5" t="inlineStr">
@@ -24934,7 +24942,7 @@
       </c>
       <c r="M185" s="5" t="inlineStr">
         <is>
-          <t>clean, fresh, soft, cool, zesty</t>
+          <t>clean, fresh, soft, zesty</t>
         </is>
       </c>
       <c r="N185" s="5" t="n"/>
@@ -25079,7 +25087,7 @@
       </c>
       <c r="M186" s="5" t="inlineStr">
         <is>
-          <t>warm, deep, cozy, sweet, sensual</t>
+          <t>warm, deep, sweet, sensual</t>
         </is>
       </c>
       <c r="N186" s="5" t="n"/>
@@ -25214,17 +25222,17 @@
       <c r="J187" s="6" t="n"/>
       <c r="K187" s="5" t="inlineStr">
         <is>
-          <t>fruity</t>
+          <t>floral</t>
         </is>
       </c>
       <c r="L187" s="5" t="inlineStr">
         <is>
-          <t>floral</t>
+          <t>citrus</t>
         </is>
       </c>
       <c r="M187" s="5" t="inlineStr">
         <is>
-          <t>fresh, lovely, zesty, sweet</t>
+          <t>fresh, soft, lovely, elegant</t>
         </is>
       </c>
       <c r="N187" s="5" t="n"/>
@@ -25733,7 +25741,7 @@
       </c>
       <c r="N191" s="5" t="inlineStr">
         <is>
-          <t>heavyFloral</t>
+          <t>heavyFloral, spicy</t>
         </is>
       </c>
       <c r="O191" s="5" t="inlineStr">
@@ -26002,12 +26010,12 @@
       </c>
       <c r="M193" s="5" t="inlineStr">
         <is>
-          <t>deep, sensual, warm</t>
+          <t>sweet, warm, sensual, deep</t>
         </is>
       </c>
       <c r="N193" s="5" t="inlineStr">
         <is>
-          <t>smoky</t>
+          <t>tooSweet</t>
         </is>
       </c>
       <c r="O193" s="5" t="inlineStr">
@@ -26139,7 +26147,7 @@
       </c>
       <c r="M194" s="5" t="inlineStr">
         <is>
-          <t>elegant, sensual, warm</t>
+          <t>elegant, sensual, warm, sweet</t>
         </is>
       </c>
       <c r="N194" s="5" t="inlineStr">
@@ -26268,7 +26276,7 @@
       </c>
       <c r="M195" s="5" t="inlineStr">
         <is>
-          <t>zesty, lovely, soft, fresh, sweet</t>
+          <t>fresh, zesty, soft, sweet</t>
         </is>
       </c>
       <c r="N195" s="5" t="n"/>
@@ -26393,12 +26401,12 @@
       </c>
       <c r="M196" s="5" t="inlineStr">
         <is>
-          <t>soft, cozy, lovely, calm, clean</t>
+          <t>soft, cozy, sweet, lovely</t>
         </is>
       </c>
       <c r="N196" s="5" t="inlineStr">
         <is>
-          <t>powdery</t>
+          <t>powdery, tooSweet</t>
         </is>
       </c>
       <c r="O196" s="5" t="inlineStr">
@@ -26925,7 +26933,7 @@
       </c>
       <c r="M200" s="5" t="inlineStr">
         <is>
-          <t>cozy, warm, sweet, sensual</t>
+          <t>cozy, warm, sweet, soft</t>
         </is>
       </c>
       <c r="N200" s="5" t="n"/>
@@ -27058,7 +27066,7 @@
       </c>
       <c r="M201" s="5" t="inlineStr">
         <is>
-          <t>lovely, fresh, soft, elegant</t>
+          <t>lovely, fresh, soft</t>
         </is>
       </c>
       <c r="N201" s="5" t="n"/>
@@ -27320,7 +27328,7 @@
       </c>
       <c r="M203" s="5" t="inlineStr">
         <is>
-          <t>fresh, elegant, zesty, sweet, lovely</t>
+          <t>fresh, zesty, elegant, sweet</t>
         </is>
       </c>
       <c r="N203" s="5" t="n"/>
@@ -27457,7 +27465,7 @@
       </c>
       <c r="M204" s="5" t="inlineStr">
         <is>
-          <t>fresh, deep, warm, calm</t>
+          <t>fresh, warm, deep</t>
         </is>
       </c>
       <c r="N204" s="5" t="inlineStr">
@@ -28150,7 +28158,7 @@
       </c>
       <c r="M209" s="5" t="inlineStr">
         <is>
-          <t>deep, sensual, warm, cozy, sweet</t>
+          <t>deep, sensual, warm, elegant</t>
         </is>
       </c>
       <c r="N209" s="5" t="inlineStr">
@@ -28412,7 +28420,7 @@
       </c>
       <c r="M211" s="5" t="inlineStr">
         <is>
-          <t>warm, sensual, elegant, cozy, sweet, deep</t>
+          <t>warm, sweet, sensual, cozy, deep</t>
         </is>
       </c>
       <c r="N211" s="5" t="inlineStr">
@@ -28549,7 +28557,7 @@
       </c>
       <c r="M212" s="5" t="inlineStr">
         <is>
-          <t>soft, cozy, calm, clean</t>
+          <t>soft, cozy, calm, warm</t>
         </is>
       </c>
       <c r="N212" s="5" t="n"/>
@@ -28560,7 +28568,7 @@
       </c>
       <c r="P212" s="5" t="inlineStr">
         <is>
-          <t>mid</t>
+          <t>high</t>
         </is>
       </c>
       <c r="Q212" s="5" t="inlineStr">
@@ -28670,7 +28678,7 @@
       </c>
       <c r="M213" s="5" t="inlineStr">
         <is>
-          <t>clean, fresh, soft, calm, cozy</t>
+          <t>clean, fresh, soft, calm</t>
         </is>
       </c>
       <c r="N213" s="5" t="n"/>

</xml_diff>

<commit_message>
tune store search queries per brand, add oliveyoung brand list and update imgs
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/perfumes-draft.xlsx
+++ b/docs/perfumes-draft.xlsx
@@ -1079,12 +1079,12 @@
       <c r="X2" s="6" t="n"/>
       <c r="Y2" s="4" t="inlineStr">
         <is>
-          <t>아쿠아 디 파르마 백화점</t>
+          <t>아쿠아디파르마</t>
         </is>
       </c>
       <c r="Z2" s="6" t="inlineStr">
         <is>
-          <t>면세점</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="AA2" s="6" t="inlineStr">
@@ -1109,7 +1109,7 @@
       </c>
       <c r="AE2" s="6" t="inlineStr">
         <is>
-          <t>낮음 (앱에 표시 안 함)</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -1212,7 +1212,7 @@
       <c r="X3" s="6" t="n"/>
       <c r="Y3" s="4" t="inlineStr">
         <is>
-          <t>톰 포드 뷰티 백화점</t>
+          <t>톰 포드 백화점</t>
         </is>
       </c>
       <c r="Z3" s="6" t="inlineStr">
@@ -1466,12 +1466,12 @@
       <c r="X5" s="6" t="n"/>
       <c r="Y5" s="4" t="inlineStr">
         <is>
-          <t>캘빈클라인 향수 백화점</t>
+          <t>올리브영 향수</t>
         </is>
       </c>
       <c r="Z5" s="6" t="inlineStr">
         <is>
-          <t>[확인 필요]</t>
+          <t>올리브영</t>
         </is>
       </c>
       <c r="AA5" s="6" t="n"/>
@@ -1488,7 +1488,7 @@
       </c>
       <c r="AE5" s="6" t="inlineStr">
         <is>
-          <t>미확인</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -1591,7 +1591,7 @@
       <c r="X6" s="6" t="n"/>
       <c r="Y6" s="4" t="inlineStr">
         <is>
-          <t>조말론 런던 백화점</t>
+          <t>조말론런던</t>
         </is>
       </c>
       <c r="Z6" s="6" t="inlineStr">
@@ -1857,12 +1857,12 @@
       </c>
       <c r="Y8" s="4" t="inlineStr">
         <is>
-          <t>버버리 향수 백화점</t>
+          <t>버버리 백화점</t>
         </is>
       </c>
       <c r="Z8" s="6" t="inlineStr">
         <is>
-          <t>[확인 필요]</t>
+          <t>올리브영</t>
         </is>
       </c>
       <c r="AA8" s="6" t="inlineStr">
@@ -1887,7 +1887,7 @@
       </c>
       <c r="AE8" s="6" t="inlineStr">
         <is>
-          <t>미확인</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -1990,7 +1990,7 @@
       <c r="X9" s="6" t="n"/>
       <c r="Y9" s="4" t="inlineStr">
         <is>
-          <t>마크제이콥스 데이지 백화점</t>
+          <t>마크제이콥스</t>
         </is>
       </c>
       <c r="Z9" s="6" t="inlineStr">
@@ -2115,7 +2115,7 @@
       <c r="X10" s="6" t="n"/>
       <c r="Y10" s="4" t="inlineStr">
         <is>
-          <t>조르지오 아르마니 뷰티 백화점</t>
+          <t>조르지오 아르마니 백화점</t>
         </is>
       </c>
       <c r="Z10" s="6" t="inlineStr">
@@ -2240,12 +2240,12 @@
       <c r="X11" s="6" t="n"/>
       <c r="Y11" s="4" t="inlineStr">
         <is>
-          <t>다비도프 쿨워터 백화점</t>
+          <t>올리브영 향수</t>
         </is>
       </c>
       <c r="Z11" s="6" t="inlineStr">
         <is>
-          <t>[확인 필요]</t>
+          <t>올리브영</t>
         </is>
       </c>
       <c r="AA11" s="6" t="n"/>
@@ -2262,7 +2262,7 @@
       </c>
       <c r="AE11" s="6" t="inlineStr">
         <is>
-          <t>미확인</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -2365,7 +2365,7 @@
       <c r="X12" s="6" t="n"/>
       <c r="Y12" s="4" t="inlineStr">
         <is>
-          <t>조말론 런던 백화점</t>
+          <t>조말론런던</t>
         </is>
       </c>
       <c r="Z12" s="6" t="inlineStr">
@@ -2490,7 +2490,7 @@
       <c r="X13" s="6" t="n"/>
       <c r="Y13" s="4" t="inlineStr">
         <is>
-          <t>조르지오 아르마니 뷰티 백화점</t>
+          <t>조르지오 아르마니 백화점</t>
         </is>
       </c>
       <c r="Z13" s="6" t="inlineStr">
@@ -2615,7 +2615,7 @@
       <c r="X14" s="6" t="n"/>
       <c r="Y14" s="4" t="inlineStr">
         <is>
-          <t>딥티크 백화점</t>
+          <t>Diptyque 백화점</t>
         </is>
       </c>
       <c r="Z14" s="6" t="inlineStr">
@@ -2740,12 +2740,12 @@
       <c r="X15" s="6" t="n"/>
       <c r="Y15" s="4" t="inlineStr">
         <is>
-          <t>에르메스 뷰티 백화점</t>
+          <t>에르메스 향수</t>
         </is>
       </c>
       <c r="Z15" s="6" t="inlineStr">
         <is>
-          <t>면세점</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="AA15" s="6" t="n"/>
@@ -2762,7 +2762,7 @@
       </c>
       <c r="AE15" s="6" t="inlineStr">
         <is>
-          <t>낮음 (앱에 표시 안 함)</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -2865,7 +2865,7 @@
       <c r="X16" s="6" t="n"/>
       <c r="Y16" s="4" t="inlineStr">
         <is>
-          <t>불가리 향수 백화점</t>
+          <t>불가리 백화점</t>
         </is>
       </c>
       <c r="Z16" s="6" t="inlineStr">
@@ -2994,7 +2994,7 @@
       <c r="X17" s="6" t="n"/>
       <c r="Y17" s="4" t="inlineStr">
         <is>
-          <t>디올 뷰티 백화점</t>
+          <t>디올 백화점</t>
         </is>
       </c>
       <c r="Z17" s="6" t="inlineStr">
@@ -3248,7 +3248,7 @@
       <c r="X19" s="6" t="n"/>
       <c r="Y19" s="4" t="inlineStr">
         <is>
-          <t>장폴고티에 향수 백화점</t>
+          <t>백화점 향수</t>
         </is>
       </c>
       <c r="Z19" s="6" t="inlineStr">
@@ -3377,7 +3377,7 @@
       <c r="X20" s="6" t="n"/>
       <c r="Y20" s="4" t="inlineStr">
         <is>
-          <t>빅터앤롤프 플라워밤 백화점</t>
+          <t>백화점 향수</t>
         </is>
       </c>
       <c r="Z20" s="6" t="inlineStr">
@@ -3502,7 +3502,7 @@
       <c r="X21" s="6" t="n"/>
       <c r="Y21" s="4" t="inlineStr">
         <is>
-          <t>디올 뷰티 백화점</t>
+          <t>디올 백화점</t>
         </is>
       </c>
       <c r="Z21" s="6" t="inlineStr">
@@ -3627,7 +3627,7 @@
       <c r="X22" s="6" t="n"/>
       <c r="Y22" s="4" t="inlineStr">
         <is>
-          <t>조말론 런던 백화점</t>
+          <t>조말론런던</t>
         </is>
       </c>
       <c r="Z22" s="6" t="inlineStr">
@@ -3877,7 +3877,7 @@
       <c r="X24" s="6" t="n"/>
       <c r="Y24" s="4" t="inlineStr">
         <is>
-          <t>디올 뷰티 백화점</t>
+          <t>디올 백화점</t>
         </is>
       </c>
       <c r="Z24" s="6" t="inlineStr">
@@ -4006,7 +4006,7 @@
       <c r="X25" s="6" t="n"/>
       <c r="Y25" s="4" t="inlineStr">
         <is>
-          <t>구찌 뷰티 백화점</t>
+          <t>구찌 향수</t>
         </is>
       </c>
       <c r="Z25" s="6" t="inlineStr">
@@ -4135,7 +4135,7 @@
       <c r="X26" s="6" t="n"/>
       <c r="Y26" s="4" t="inlineStr">
         <is>
-          <t>딥티크 백화점</t>
+          <t>Diptyque 백화점</t>
         </is>
       </c>
       <c r="Z26" s="6" t="inlineStr">
@@ -4393,7 +4393,7 @@
       <c r="X28" s="6" t="n"/>
       <c r="Y28" s="4" t="inlineStr">
         <is>
-          <t>프라다 뷰티 백화점</t>
+          <t>프라다 백화점</t>
         </is>
       </c>
       <c r="Z28" s="6" t="inlineStr">
@@ -4522,7 +4522,7 @@
       <c r="X29" s="6" t="n"/>
       <c r="Y29" s="4" t="inlineStr">
         <is>
-          <t>디올 뷰티 백화점</t>
+          <t>디올 백화점</t>
         </is>
       </c>
       <c r="Z29" s="6" t="inlineStr">
@@ -4651,12 +4651,12 @@
       <c r="X30" s="6" t="n"/>
       <c r="Y30" s="4" t="inlineStr">
         <is>
-          <t>끌로에 향수 백화점</t>
+          <t>끌로에 백화점</t>
         </is>
       </c>
       <c r="Z30" s="6" t="inlineStr">
         <is>
-          <t>[확인 필요]</t>
+          <t>올리브영</t>
         </is>
       </c>
       <c r="AA30" s="6" t="n"/>
@@ -4673,7 +4673,7 @@
       </c>
       <c r="AE30" s="6" t="inlineStr">
         <is>
-          <t>미확인</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -4792,12 +4792,12 @@
       </c>
       <c r="Y31" s="4" t="inlineStr">
         <is>
-          <t>바이레도 백화점</t>
+          <t>바이레도</t>
         </is>
       </c>
       <c r="Z31" s="6" t="inlineStr">
         <is>
-          <t>[확인 필요]</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="AA31" s="6" t="inlineStr">
@@ -4822,7 +4822,7 @@
       </c>
       <c r="AE31" s="6" t="inlineStr">
         <is>
-          <t>미확인</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -4941,7 +4941,7 @@
       </c>
       <c r="Y32" s="4" t="inlineStr">
         <is>
-          <t>메종 마르지엘라 레플리카 백화점</t>
+          <t>메종 마르지엘라 향수</t>
         </is>
       </c>
       <c r="Z32" s="6" t="inlineStr">
@@ -5074,7 +5074,7 @@
       <c r="X33" s="6" t="n"/>
       <c r="Y33" s="4" t="inlineStr">
         <is>
-          <t>나르시소 로드리게즈 백화점</t>
+          <t>올리브영 향수</t>
         </is>
       </c>
       <c r="Z33" s="6" t="inlineStr">
@@ -5203,7 +5203,7 @@
       <c r="X34" s="6" t="n"/>
       <c r="Y34" s="4" t="inlineStr">
         <is>
-          <t>딥티크 백화점</t>
+          <t>Diptyque 백화점</t>
         </is>
       </c>
       <c r="Z34" s="6" t="inlineStr">
@@ -5328,7 +5328,7 @@
       <c r="X35" s="6" t="n"/>
       <c r="Y35" s="4" t="inlineStr">
         <is>
-          <t>메종 마르지엘라 레플리카 백화점</t>
+          <t>메종 마르지엘라 향수</t>
         </is>
       </c>
       <c r="Z35" s="6" t="inlineStr">
@@ -5457,12 +5457,12 @@
       <c r="X36" s="6" t="n"/>
       <c r="Y36" s="4" t="inlineStr">
         <is>
-          <t>에르메스 뷰티 백화점</t>
+          <t>에르메스 향수</t>
         </is>
       </c>
       <c r="Z36" s="6" t="inlineStr">
         <is>
-          <t>면세점</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="AA36" s="6" t="n"/>
@@ -5479,7 +5479,7 @@
       </c>
       <c r="AE36" s="6" t="inlineStr">
         <is>
-          <t>낮음 (앱에 표시 안 함)</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -5586,12 +5586,12 @@
       <c r="X37" s="6" t="n"/>
       <c r="Y37" s="4" t="inlineStr">
         <is>
-          <t>에르메스 뷰티 백화점</t>
+          <t>에르메스 향수</t>
         </is>
       </c>
       <c r="Z37" s="6" t="inlineStr">
         <is>
-          <t>면세점</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="AA37" s="6" t="n"/>
@@ -5608,7 +5608,7 @@
       </c>
       <c r="AE37" s="6" t="inlineStr">
         <is>
-          <t>낮음 (앱에 표시 안 함)</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -5727,7 +5727,7 @@
       </c>
       <c r="Y38" s="4" t="inlineStr">
         <is>
-          <t>르 라보 백화점</t>
+          <t>르 라보 성수</t>
         </is>
       </c>
       <c r="Z38" s="6" t="inlineStr">
@@ -5860,7 +5860,7 @@
       <c r="X39" s="6" t="n"/>
       <c r="Y39" s="4" t="inlineStr">
         <is>
-          <t>딥티크 백화점</t>
+          <t>Diptyque 백화점</t>
         </is>
       </c>
       <c r="Z39" s="6" t="inlineStr">
@@ -5989,7 +5989,7 @@
       <c r="X40" s="6" t="n"/>
       <c r="Y40" s="4" t="inlineStr">
         <is>
-          <t>톰 포드 뷰티 백화점</t>
+          <t>톰 포드 백화점</t>
         </is>
       </c>
       <c r="Z40" s="6" t="inlineStr">
@@ -6126,12 +6126,12 @@
       </c>
       <c r="Y41" s="4" t="inlineStr">
         <is>
-          <t>바이레도 백화점</t>
+          <t>바이레도</t>
         </is>
       </c>
       <c r="Z41" s="6" t="inlineStr">
         <is>
-          <t>[확인 필요]</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="AA41" s="6" t="inlineStr">
@@ -6156,7 +6156,7 @@
       </c>
       <c r="AE41" s="6" t="inlineStr">
         <is>
-          <t>미확인</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -6263,7 +6263,7 @@
       <c r="X42" s="6" t="n"/>
       <c r="Y42" s="4" t="inlineStr">
         <is>
-          <t>메종 프란시스 커정 백화점</t>
+          <t>메종프란시스커정</t>
         </is>
       </c>
       <c r="Z42" s="6" t="inlineStr">
@@ -6392,7 +6392,7 @@
       <c r="X43" s="6" t="n"/>
       <c r="Y43" s="4" t="inlineStr">
         <is>
-          <t>겔랑 향수 백화점</t>
+          <t>겔랑</t>
         </is>
       </c>
       <c r="Z43" s="6" t="inlineStr">
@@ -6517,7 +6517,7 @@
       <c r="X44" s="6" t="n"/>
       <c r="Y44" s="4" t="inlineStr">
         <is>
-          <t>입생로랑 뷰티 백화점</t>
+          <t>입생로랑 백화점</t>
         </is>
       </c>
       <c r="Z44" s="6" t="inlineStr">
@@ -6646,7 +6646,7 @@
       <c r="X45" s="6" t="n"/>
       <c r="Y45" s="4" t="inlineStr">
         <is>
-          <t>입생로랑 뷰티 백화점</t>
+          <t>입생로랑 백화점</t>
         </is>
       </c>
       <c r="Z45" s="6" t="inlineStr">
@@ -6775,12 +6775,12 @@
       <c r="X46" s="6" t="n"/>
       <c r="Y46" s="4" t="inlineStr">
         <is>
-          <t>랑콤 뷰티 백화점</t>
+          <t>랑콤 백화점</t>
         </is>
       </c>
       <c r="Z46" s="6" t="inlineStr">
         <is>
-          <t>백화점</t>
+          <t>백화점, 올리브영</t>
         </is>
       </c>
       <c r="AA46" s="6" t="n"/>
@@ -6904,7 +6904,7 @@
       <c r="X47" s="6" t="n"/>
       <c r="Y47" s="4" t="inlineStr">
         <is>
-          <t>킬리안 파리 백화점</t>
+          <t>킬리안 백화점</t>
         </is>
       </c>
       <c r="Z47" s="6" t="inlineStr">
@@ -6926,7 +6926,7 @@
       </c>
       <c r="AE47" s="6" t="inlineStr">
         <is>
-          <t>낮음 (앱에 표시 안 함)</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -7033,7 +7033,7 @@
       <c r="X48" s="6" t="n"/>
       <c r="Y48" s="4" t="inlineStr">
         <is>
-          <t>뮈글러 엔젤 백화점</t>
+          <t>백화점 향수</t>
         </is>
       </c>
       <c r="Z48" s="6" t="inlineStr">
@@ -7174,7 +7174,7 @@
       </c>
       <c r="Y49" s="4" t="inlineStr">
         <is>
-          <t>메종 마르지엘라 레플리카 백화점</t>
+          <t>메종 마르지엘라 향수</t>
         </is>
       </c>
       <c r="Z49" s="6" t="inlineStr">
@@ -7311,7 +7311,7 @@
       <c r="X50" s="6" t="n"/>
       <c r="Y50" s="4" t="inlineStr">
         <is>
-          <t>메종 마르지엘라 레플리카 백화점</t>
+          <t>메종 마르지엘라 향수</t>
         </is>
       </c>
       <c r="Z50" s="6" t="inlineStr">
@@ -7440,7 +7440,7 @@
       <c r="X51" s="6" t="n"/>
       <c r="Y51" s="4" t="inlineStr">
         <is>
-          <t>톰 포드 뷰티 백화점</t>
+          <t>톰 포드 백화점</t>
         </is>
       </c>
       <c r="Z51" s="6" t="inlineStr">
@@ -7577,7 +7577,7 @@
       </c>
       <c r="Y52" s="4" t="inlineStr">
         <is>
-          <t>르 라보 백화점</t>
+          <t>르 라보 성수</t>
         </is>
       </c>
       <c r="Z52" s="6" t="inlineStr">
@@ -7726,7 +7726,7 @@
       </c>
       <c r="Y53" s="4" t="inlineStr">
         <is>
-          <t>르 라보 백화점</t>
+          <t>르 라보 성수</t>
         </is>
       </c>
       <c r="Z53" s="6" t="inlineStr">
@@ -7875,7 +7875,7 @@
       </c>
       <c r="Y54" s="4" t="inlineStr">
         <is>
-          <t>르 라보 백화점</t>
+          <t>르 라보 성수</t>
         </is>
       </c>
       <c r="Z54" s="6" t="inlineStr">
@@ -8020,7 +8020,7 @@
       </c>
       <c r="Y55" s="4" t="inlineStr">
         <is>
-          <t>르 라보 백화점</t>
+          <t>르 라보 성수</t>
         </is>
       </c>
       <c r="Z55" s="6" t="inlineStr">
@@ -8157,7 +8157,7 @@
       <c r="X56" s="6" t="n"/>
       <c r="Y56" s="4" t="inlineStr">
         <is>
-          <t>킬리안 파리 백화점</t>
+          <t>킬리안 백화점</t>
         </is>
       </c>
       <c r="Z56" s="6" t="inlineStr">
@@ -8179,7 +8179,7 @@
       </c>
       <c r="AE56" s="6" t="inlineStr">
         <is>
-          <t>낮음 (앱에 표시 안 함)</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -8286,7 +8286,7 @@
       <c r="X57" s="6" t="n"/>
       <c r="Y57" s="4" t="inlineStr">
         <is>
-          <t>킬리안 파리 백화점</t>
+          <t>킬리안 백화점</t>
         </is>
       </c>
       <c r="Z57" s="6" t="inlineStr">
@@ -8308,7 +8308,7 @@
       </c>
       <c r="AE57" s="6" t="inlineStr">
         <is>
-          <t>낮음 (앱에 표시 안 함)</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -8415,12 +8415,12 @@
       <c r="X58" s="6" t="n"/>
       <c r="Y58" s="4" t="inlineStr">
         <is>
-          <t>크리드 백화점</t>
+          <t>크리드 향수</t>
         </is>
       </c>
       <c r="Z58" s="6" t="inlineStr">
         <is>
-          <t>면세점</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="AA58" s="6" t="n"/>
@@ -8437,7 +8437,7 @@
       </c>
       <c r="AE58" s="6" t="inlineStr">
         <is>
-          <t>낮음 (앱에 표시 안 함)</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -8540,12 +8540,12 @@
       <c r="X59" s="6" t="n"/>
       <c r="Y59" s="4" t="inlineStr">
         <is>
-          <t>크리드 백화점</t>
+          <t>크리드 향수</t>
         </is>
       </c>
       <c r="Z59" s="6" t="inlineStr">
         <is>
-          <t>면세점</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="AA59" s="6" t="n"/>
@@ -8562,7 +8562,7 @@
       </c>
       <c r="AE59" s="6" t="inlineStr">
         <is>
-          <t>낮음 (앱에 표시 안 함)</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -8665,12 +8665,12 @@
       <c r="X60" s="6" t="n"/>
       <c r="Y60" s="4" t="inlineStr">
         <is>
-          <t>크리드 백화점</t>
+          <t>크리드 향수</t>
         </is>
       </c>
       <c r="Z60" s="6" t="inlineStr">
         <is>
-          <t>면세점</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="AA60" s="6" t="n"/>
@@ -8687,7 +8687,7 @@
       </c>
       <c r="AE60" s="6" t="inlineStr">
         <is>
-          <t>낮음 (앱에 표시 안 함)</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -8790,12 +8790,12 @@
       <c r="X61" s="6" t="n"/>
       <c r="Y61" s="4" t="inlineStr">
         <is>
-          <t>크리드 백화점</t>
+          <t>크리드 향수</t>
         </is>
       </c>
       <c r="Z61" s="6" t="inlineStr">
         <is>
-          <t>면세점</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="AA61" s="6" t="n"/>
@@ -8812,7 +8812,7 @@
       </c>
       <c r="AE61" s="6" t="inlineStr">
         <is>
-          <t>낮음 (앱에 표시 안 함)</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -8924,7 +8924,7 @@
       </c>
       <c r="Z62" s="6" t="inlineStr">
         <is>
-          <t>면세점</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="AA62" s="6" t="n"/>
@@ -8941,7 +8941,7 @@
       </c>
       <c r="AE62" s="6" t="inlineStr">
         <is>
-          <t>낮음 (앱에 표시 안 함)</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -9053,7 +9053,7 @@
       </c>
       <c r="Z63" s="6" t="inlineStr">
         <is>
-          <t>면세점</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="AA63" s="6" t="n"/>
@@ -9070,7 +9070,7 @@
       </c>
       <c r="AE63" s="6" t="inlineStr">
         <is>
-          <t>낮음 (앱에 표시 안 함)</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -9182,7 +9182,7 @@
       </c>
       <c r="Z64" s="6" t="inlineStr">
         <is>
-          <t>면세점</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="AA64" s="6" t="n"/>
@@ -9199,7 +9199,7 @@
       </c>
       <c r="AE64" s="6" t="inlineStr">
         <is>
-          <t>낮음 (앱에 표시 안 함)</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -9311,7 +9311,7 @@
       </c>
       <c r="Z65" s="6" t="inlineStr">
         <is>
-          <t>면세점</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="AA65" s="6" t="n"/>
@@ -9328,7 +9328,7 @@
       </c>
       <c r="AE65" s="6" t="inlineStr">
         <is>
-          <t>낮음 (앱에 표시 안 함)</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -9440,7 +9440,7 @@
       </c>
       <c r="Z66" s="6" t="inlineStr">
         <is>
-          <t>면세점</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="AA66" s="6" t="n"/>
@@ -9457,7 +9457,7 @@
       </c>
       <c r="AE66" s="6" t="inlineStr">
         <is>
-          <t>낮음 (앱에 표시 안 함)</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -9560,7 +9560,7 @@
       <c r="X67" s="6" t="n"/>
       <c r="Y67" s="4" t="inlineStr">
         <is>
-          <t>아닉 구딸 백화점</t>
+          <t>백화점 향수</t>
         </is>
       </c>
       <c r="Z67" s="6" t="inlineStr">
@@ -9685,7 +9685,7 @@
       <c r="X68" s="6" t="n"/>
       <c r="Y68" s="4" t="inlineStr">
         <is>
-          <t>아닉 구딸 백화점</t>
+          <t>백화점 향수</t>
         </is>
       </c>
       <c r="Z68" s="6" t="inlineStr">
@@ -10104,12 +10104,12 @@
       <c r="X71" s="6" t="n"/>
       <c r="Y71" s="4" t="inlineStr">
         <is>
-          <t>퍼퓸 드 말리 백화점</t>
+          <t>퍼퓸드말리</t>
         </is>
       </c>
       <c r="Z71" s="6" t="inlineStr">
         <is>
-          <t>[확인 필요]</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="AA71" s="6" t="n"/>
@@ -10126,7 +10126,7 @@
       </c>
       <c r="AE71" s="6" t="inlineStr">
         <is>
-          <t>미확인</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -10233,12 +10233,12 @@
       <c r="X72" s="6" t="n"/>
       <c r="Y72" s="4" t="inlineStr">
         <is>
-          <t>퍼퓸 드 말리 백화점</t>
+          <t>퍼퓸드말리</t>
         </is>
       </c>
       <c r="Z72" s="6" t="inlineStr">
         <is>
-          <t>[확인 필요]</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="AA72" s="6" t="n"/>
@@ -10255,7 +10255,7 @@
       </c>
       <c r="AE72" s="6" t="inlineStr">
         <is>
-          <t>미확인</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -10362,7 +10362,7 @@
       <c r="X73" s="6" t="n"/>
       <c r="Y73" s="4" t="inlineStr">
         <is>
-          <t>메종 프란시스 커정 백화점</t>
+          <t>메종프란시스커정</t>
         </is>
       </c>
       <c r="Z73" s="6" t="inlineStr">
@@ -10487,7 +10487,7 @@
       <c r="X74" s="6" t="n"/>
       <c r="Y74" s="4" t="inlineStr">
         <is>
-          <t>메종 프란시스 커정 백화점</t>
+          <t>메종프란시스커정</t>
         </is>
       </c>
       <c r="Z74" s="6" t="inlineStr">
@@ -10616,7 +10616,7 @@
       <c r="X75" s="6" t="n"/>
       <c r="Y75" s="4" t="inlineStr">
         <is>
-          <t>메종 프란시스 커정 백화점</t>
+          <t>메종프란시스커정</t>
         </is>
       </c>
       <c r="Z75" s="6" t="inlineStr">
@@ -10741,7 +10741,7 @@
       <c r="X76" s="6" t="n"/>
       <c r="Y76" s="4" t="inlineStr">
         <is>
-          <t>메종 프란시스 커정 백화점</t>
+          <t>메종프란시스커정</t>
         </is>
       </c>
       <c r="Z76" s="6" t="inlineStr">
@@ -10870,7 +10870,7 @@
       <c r="X77" s="6" t="n"/>
       <c r="Y77" s="4" t="inlineStr">
         <is>
-          <t>이니시오 백화점</t>
+          <t>백화점 향수</t>
         </is>
       </c>
       <c r="Z77" s="6" t="inlineStr">
@@ -10995,12 +10995,12 @@
       <c r="X78" s="6" t="n"/>
       <c r="Y78" s="4" t="inlineStr">
         <is>
-          <t>니샤네 백화점</t>
+          <t>퍼퓸갤러리</t>
         </is>
       </c>
       <c r="Z78" s="6" t="inlineStr">
         <is>
-          <t>[확인 필요]</t>
+          <t>편집숍(퍼퓸갤러리)</t>
         </is>
       </c>
       <c r="AA78" s="6" t="n"/>
@@ -11017,7 +11017,7 @@
       </c>
       <c r="AE78" s="6" t="inlineStr">
         <is>
-          <t>미확인</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -11136,12 +11136,12 @@
       </c>
       <c r="Y79" s="4" t="inlineStr">
         <is>
-          <t>바이레도 백화점</t>
+          <t>바이레도</t>
         </is>
       </c>
       <c r="Z79" s="6" t="inlineStr">
         <is>
-          <t>[확인 필요]</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="AA79" s="6" t="inlineStr">
@@ -11166,7 +11166,7 @@
       </c>
       <c r="AE79" s="6" t="inlineStr">
         <is>
-          <t>미확인</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -11281,12 +11281,12 @@
       </c>
       <c r="Y80" s="4" t="inlineStr">
         <is>
-          <t>바이레도 백화점</t>
+          <t>바이레도</t>
         </is>
       </c>
       <c r="Z80" s="6" t="inlineStr">
         <is>
-          <t>[확인 필요]</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="AA80" s="6" t="inlineStr">
@@ -11311,7 +11311,7 @@
       </c>
       <c r="AE80" s="6" t="inlineStr">
         <is>
-          <t>미확인</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -11426,12 +11426,12 @@
       </c>
       <c r="Y81" s="4" t="inlineStr">
         <is>
-          <t>바이레도 백화점</t>
+          <t>바이레도</t>
         </is>
       </c>
       <c r="Z81" s="6" t="inlineStr">
         <is>
-          <t>[확인 필요]</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="AA81" s="6" t="inlineStr">
@@ -11456,7 +11456,7 @@
       </c>
       <c r="AE81" s="6" t="inlineStr">
         <is>
-          <t>미확인</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -11571,12 +11571,12 @@
       </c>
       <c r="Y82" s="4" t="inlineStr">
         <is>
-          <t>바이레도 백화점</t>
+          <t>바이레도</t>
         </is>
       </c>
       <c r="Z82" s="6" t="inlineStr">
         <is>
-          <t>[확인 필요]</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="AA82" s="6" t="inlineStr">
@@ -11601,7 +11601,7 @@
       </c>
       <c r="AE82" s="6" t="inlineStr">
         <is>
-          <t>미확인</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -11708,7 +11708,7 @@
       <c r="X83" s="6" t="n"/>
       <c r="Y83" s="4" t="inlineStr">
         <is>
-          <t>딥티크 백화점</t>
+          <t>Diptyque 백화점</t>
         </is>
       </c>
       <c r="Z83" s="6" t="inlineStr">
@@ -11833,7 +11833,7 @@
       <c r="X84" s="6" t="n"/>
       <c r="Y84" s="4" t="inlineStr">
         <is>
-          <t>딥티크 백화점</t>
+          <t>Diptyque 백화점</t>
         </is>
       </c>
       <c r="Z84" s="6" t="inlineStr">
@@ -11962,7 +11962,7 @@
       <c r="X85" s="6" t="n"/>
       <c r="Y85" s="4" t="inlineStr">
         <is>
-          <t>톰 포드 뷰티 백화점</t>
+          <t>톰 포드 백화점</t>
         </is>
       </c>
       <c r="Z85" s="6" t="inlineStr">
@@ -12087,7 +12087,7 @@
       <c r="X86" s="6" t="n"/>
       <c r="Y86" s="4" t="inlineStr">
         <is>
-          <t>톰 포드 뷰티 백화점</t>
+          <t>톰 포드 백화점</t>
         </is>
       </c>
       <c r="Z86" s="6" t="inlineStr">
@@ -12216,7 +12216,7 @@
       <c r="X87" s="6" t="n"/>
       <c r="Y87" s="4" t="inlineStr">
         <is>
-          <t>톰 포드 뷰티 백화점</t>
+          <t>톰 포드 백화점</t>
         </is>
       </c>
       <c r="Z87" s="6" t="inlineStr">
@@ -12345,7 +12345,7 @@
       <c r="X88" s="6" t="n"/>
       <c r="Y88" s="4" t="inlineStr">
         <is>
-          <t>톰 포드 뷰티 백화점</t>
+          <t>톰 포드 백화점</t>
         </is>
       </c>
       <c r="Z88" s="6" t="inlineStr">
@@ -12474,7 +12474,7 @@
       <c r="X89" s="6" t="n"/>
       <c r="Y89" s="4" t="inlineStr">
         <is>
-          <t>톰 포드 뷰티 백화점</t>
+          <t>톰 포드 백화점</t>
         </is>
       </c>
       <c r="Z89" s="6" t="inlineStr">
@@ -12599,12 +12599,12 @@
       <c r="X90" s="6" t="n"/>
       <c r="Y90" s="4" t="inlineStr">
         <is>
-          <t>에르메스 뷰티 백화점</t>
+          <t>에르메스 향수</t>
         </is>
       </c>
       <c r="Z90" s="6" t="inlineStr">
         <is>
-          <t>면세점</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="AA90" s="6" t="n"/>
@@ -12621,7 +12621,7 @@
       </c>
       <c r="AE90" s="6" t="inlineStr">
         <is>
-          <t>낮음 (앱에 표시 안 함)</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -12724,12 +12724,12 @@
       <c r="X91" s="6" t="n"/>
       <c r="Y91" s="4" t="inlineStr">
         <is>
-          <t>아쿠아 디 파르마 백화점</t>
+          <t>아쿠아디파르마</t>
         </is>
       </c>
       <c r="Z91" s="6" t="inlineStr">
         <is>
-          <t>면세점</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="AA91" s="6" t="n"/>
@@ -12746,7 +12746,7 @@
       </c>
       <c r="AE91" s="6" t="inlineStr">
         <is>
-          <t>낮음 (앱에 표시 안 함)</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -12849,7 +12849,7 @@
       <c r="X92" s="6" t="n"/>
       <c r="Y92" s="4" t="inlineStr">
         <is>
-          <t>펜할리곤스 백화점</t>
+          <t>펜할리곤스</t>
         </is>
       </c>
       <c r="Z92" s="6" t="inlineStr">
@@ -12974,12 +12974,12 @@
       <c r="X93" s="6" t="n"/>
       <c r="Y93" s="4" t="inlineStr">
         <is>
-          <t>아틀리에 코롱 백화점</t>
+          <t>아틀리에 코롱</t>
         </is>
       </c>
       <c r="Z93" s="6" t="inlineStr">
         <is>
-          <t>[확인 필요]</t>
+          <t>백화점</t>
         </is>
       </c>
       <c r="AA93" s="6" t="n"/>
@@ -12996,7 +12996,7 @@
       </c>
       <c r="AE93" s="6" t="inlineStr">
         <is>
-          <t>미확인</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -13103,12 +13103,12 @@
       <c r="X94" s="6" t="n"/>
       <c r="Y94" s="4" t="inlineStr">
         <is>
-          <t>제르조프 백화점</t>
+          <t>퍼퓸갤러리</t>
         </is>
       </c>
       <c r="Z94" s="6" t="inlineStr">
         <is>
-          <t>백화점</t>
+          <t>편집숍(퍼퓸갤러리)</t>
         </is>
       </c>
       <c r="AA94" s="6" t="n"/>
@@ -13125,7 +13125,7 @@
       </c>
       <c r="AE94" s="6" t="inlineStr">
         <is>
-          <t>낮음 (앱에 표시 안 함)</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -13220,7 +13220,7 @@
       <c r="X95" s="6" t="n"/>
       <c r="Y95" s="4" t="inlineStr">
         <is>
-          <t>에센트릭 몰큘스 백화점</t>
+          <t>백화점 향수</t>
         </is>
       </c>
       <c r="Z95" s="6" t="inlineStr">
@@ -13337,7 +13337,7 @@
       <c r="X96" s="6" t="n"/>
       <c r="Y96" s="4" t="inlineStr">
         <is>
-          <t>에센트릭 몰큘스 백화점</t>
+          <t>백화점 향수</t>
         </is>
       </c>
       <c r="Z96" s="6" t="inlineStr">
@@ -13454,12 +13454,12 @@
       <c r="X97" s="6" t="n"/>
       <c r="Y97" s="4" t="inlineStr">
         <is>
-          <t>줄리엣 해즈 어 건 백화점</t>
+          <t>줄리엣 해즈 어 건</t>
         </is>
       </c>
       <c r="Z97" s="6" t="inlineStr">
         <is>
-          <t>편집숍</t>
+          <t>백화점</t>
         </is>
       </c>
       <c r="AA97" s="6" t="n"/>
@@ -13476,7 +13476,7 @@
       </c>
       <c r="AE97" s="6" t="inlineStr">
         <is>
-          <t>낮음 (앱에 표시 안 함)</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -13579,12 +13579,12 @@
       <c r="X98" s="6" t="n"/>
       <c r="Y98" s="4" t="inlineStr">
         <is>
-          <t>엑스 니힐로 백화점</t>
+          <t>엑스니힐로</t>
         </is>
       </c>
       <c r="Z98" s="6" t="inlineStr">
         <is>
-          <t>면세점</t>
+          <t>백화점</t>
         </is>
       </c>
       <c r="AA98" s="6" t="n"/>
@@ -13601,7 +13601,7 @@
       </c>
       <c r="AE98" s="6" t="inlineStr">
         <is>
-          <t>낮음 (앱에 표시 안 함)</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -13708,12 +13708,12 @@
       <c r="X99" s="6" t="n"/>
       <c r="Y99" s="4" t="inlineStr">
         <is>
-          <t>퍼퓸 드 말리 백화점</t>
+          <t>퍼퓸드말리</t>
         </is>
       </c>
       <c r="Z99" s="6" t="inlineStr">
         <is>
-          <t>[확인 필요]</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="AA99" s="6" t="n"/>
@@ -13730,7 +13730,7 @@
       </c>
       <c r="AE99" s="6" t="inlineStr">
         <is>
-          <t>미확인</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -13962,7 +13962,7 @@
       <c r="X101" s="6" t="n"/>
       <c r="Y101" s="4" t="inlineStr">
         <is>
-          <t>베르사체 향수 매장</t>
+          <t>베르사체 백화점</t>
         </is>
       </c>
       <c r="Z101" s="6" t="inlineStr">
@@ -14091,7 +14091,7 @@
       <c r="X102" s="6" t="n"/>
       <c r="Y102" s="4" t="inlineStr">
         <is>
-          <t>베르사체 향수 매장</t>
+          <t>베르사체 백화점</t>
         </is>
       </c>
       <c r="Z102" s="6" t="inlineStr">
@@ -14220,7 +14220,7 @@
       <c r="X103" s="6" t="n"/>
       <c r="Y103" s="4" t="inlineStr">
         <is>
-          <t>파코 라반 향수 매장</t>
+          <t>백화점 향수</t>
         </is>
       </c>
       <c r="Z103" s="6" t="inlineStr">
@@ -14349,7 +14349,7 @@
       <c r="X104" s="6" t="n"/>
       <c r="Y104" s="4" t="inlineStr">
         <is>
-          <t>파코 라반 향수 매장</t>
+          <t>백화점 향수</t>
         </is>
       </c>
       <c r="Z104" s="6" t="inlineStr">
@@ -14478,7 +14478,7 @@
       <c r="X105" s="6" t="n"/>
       <c r="Y105" s="4" t="inlineStr">
         <is>
-          <t>휴고 보스 향수 매장</t>
+          <t>휴고 보스 백화점</t>
         </is>
       </c>
       <c r="Z105" s="6" t="inlineStr">
@@ -14603,12 +14603,12 @@
       <c r="X106" s="6" t="n"/>
       <c r="Y106" s="4" t="inlineStr">
         <is>
-          <t>캘빈클라인 향수 매장</t>
+          <t>올리브영 향수</t>
         </is>
       </c>
       <c r="Z106" s="6" t="inlineStr">
         <is>
-          <t>[확인 필요]</t>
+          <t>올리브영</t>
         </is>
       </c>
       <c r="AA106" s="6" t="n"/>
@@ -14625,7 +14625,7 @@
       </c>
       <c r="AE106" s="6" t="inlineStr">
         <is>
-          <t>미확인</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -14732,7 +14732,7 @@
       <c r="X107" s="6" t="n"/>
       <c r="Y107" s="4" t="inlineStr">
         <is>
-          <t>캐롤리나 헤레라 향수 매장</t>
+          <t>백화점 향수</t>
         </is>
       </c>
       <c r="Z107" s="6" t="inlineStr">
@@ -14857,7 +14857,7 @@
       <c r="X108" s="6" t="n"/>
       <c r="Y108" s="4" t="inlineStr">
         <is>
-          <t>입생로랑 뷰티 백화점</t>
+          <t>입생로랑 백화점</t>
         </is>
       </c>
       <c r="Z108" s="6" t="inlineStr">
@@ -14982,12 +14982,12 @@
       <c r="X109" s="6" t="n"/>
       <c r="Y109" s="4" t="inlineStr">
         <is>
-          <t>랑콤 뷰티 백화점</t>
+          <t>랑콤 백화점</t>
         </is>
       </c>
       <c r="Z109" s="6" t="inlineStr">
         <is>
-          <t>백화점</t>
+          <t>백화점, 올리브영</t>
         </is>
       </c>
       <c r="AA109" s="6" t="n"/>
@@ -15107,7 +15107,7 @@
       <c r="X110" s="6" t="n"/>
       <c r="Y110" s="4" t="inlineStr">
         <is>
-          <t>몽블랑 향수 매장</t>
+          <t>올리브영 향수</t>
         </is>
       </c>
       <c r="Z110" s="6" t="inlineStr">
@@ -15232,7 +15232,7 @@
       <c r="X111" s="6" t="n"/>
       <c r="Y111" s="4" t="inlineStr">
         <is>
-          <t>조르지오 아르마니 뷰티 백화점</t>
+          <t>조르지오 아르마니 백화점</t>
         </is>
       </c>
       <c r="Z111" s="6" t="inlineStr">
@@ -15357,7 +15357,7 @@
       <c r="X112" s="6" t="n"/>
       <c r="Y112" s="4" t="inlineStr">
         <is>
-          <t>불가리 향수 매장</t>
+          <t>불가리 백화점</t>
         </is>
       </c>
       <c r="Z112" s="6" t="inlineStr">
@@ -15486,7 +15486,7 @@
       <c r="X113" s="6" t="n"/>
       <c r="Y113" s="4" t="inlineStr">
         <is>
-          <t>입생로랑 뷰티 백화점</t>
+          <t>입생로랑 백화점</t>
         </is>
       </c>
       <c r="Z113" s="6" t="inlineStr">
@@ -15615,7 +15615,7 @@
       <c r="X114" s="6" t="n"/>
       <c r="Y114" s="4" t="inlineStr">
         <is>
-          <t>프라다 뷰티 백화점</t>
+          <t>프라다 백화점</t>
         </is>
       </c>
       <c r="Z114" s="6" t="inlineStr">
@@ -15744,7 +15744,7 @@
       <c r="X115" s="6" t="n"/>
       <c r="Y115" s="4" t="inlineStr">
         <is>
-          <t>뮈글러 향수 매장</t>
+          <t>백화점 향수</t>
         </is>
       </c>
       <c r="Z115" s="6" t="inlineStr">
@@ -15869,7 +15869,7 @@
       <c r="X116" s="6" t="n"/>
       <c r="Y116" s="4" t="inlineStr">
         <is>
-          <t>샤넬 백화점</t>
+          <t>샤넬 뷰티 백화점</t>
         </is>
       </c>
       <c r="Z116" s="6" t="inlineStr">
@@ -15994,7 +15994,7 @@
       <c r="X117" s="6" t="n"/>
       <c r="Y117" s="4" t="inlineStr">
         <is>
-          <t>샤넬 백화점</t>
+          <t>샤넬 뷰티 백화점</t>
         </is>
       </c>
       <c r="Z117" s="6" t="inlineStr">
@@ -16119,7 +16119,7 @@
       <c r="X118" s="6" t="n"/>
       <c r="Y118" s="4" t="inlineStr">
         <is>
-          <t>샤넬 백화점</t>
+          <t>샤넬 뷰티 백화점</t>
         </is>
       </c>
       <c r="Z118" s="6" t="inlineStr">
@@ -17147,12 +17147,12 @@
       </c>
       <c r="Y126" s="4" t="inlineStr">
         <is>
-          <t>에르메스 백화점</t>
+          <t>에르메스 향수</t>
         </is>
       </c>
       <c r="Z126" s="6" t="inlineStr">
         <is>
-          <t>면세점</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="AA126" s="6" t="inlineStr">
@@ -17177,7 +17177,7 @@
       </c>
       <c r="AE126" s="6" t="inlineStr">
         <is>
-          <t>낮음 (앱에 표시 안 함)</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -17292,12 +17292,12 @@
       </c>
       <c r="Y127" s="4" t="inlineStr">
         <is>
-          <t>에르메스 백화점</t>
+          <t>에르메스 향수</t>
         </is>
       </c>
       <c r="Z127" s="6" t="inlineStr">
         <is>
-          <t>면세점</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="AA127" s="6" t="inlineStr">
@@ -17322,7 +17322,7 @@
       </c>
       <c r="AE127" s="6" t="inlineStr">
         <is>
-          <t>낮음 (앱에 표시 안 함)</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -17425,12 +17425,12 @@
       <c r="X128" s="6" t="n"/>
       <c r="Y128" s="4" t="inlineStr">
         <is>
-          <t>에르메스 백화점</t>
+          <t>에르메스 향수</t>
         </is>
       </c>
       <c r="Z128" s="6" t="inlineStr">
         <is>
-          <t>면세점</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="AA128" s="6" t="inlineStr">
@@ -17455,7 +17455,7 @@
       </c>
       <c r="AE128" s="6" t="inlineStr">
         <is>
-          <t>낮음 (앱에 표시 안 함)</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -17570,12 +17570,12 @@
       </c>
       <c r="Y129" s="4" t="inlineStr">
         <is>
-          <t>에르메스 백화점</t>
+          <t>에르메스 향수</t>
         </is>
       </c>
       <c r="Z129" s="6" t="inlineStr">
         <is>
-          <t>면세점</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="AA129" s="6" t="inlineStr">
@@ -17600,7 +17600,7 @@
       </c>
       <c r="AE129" s="6" t="inlineStr">
         <is>
-          <t>낮음 (앱에 표시 안 함)</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -17715,12 +17715,12 @@
       </c>
       <c r="Y130" s="4" t="inlineStr">
         <is>
-          <t>에르메스 백화점</t>
+          <t>에르메스 향수</t>
         </is>
       </c>
       <c r="Z130" s="6" t="inlineStr">
         <is>
-          <t>면세점</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="AA130" s="6" t="inlineStr">
@@ -17745,7 +17745,7 @@
       </c>
       <c r="AE130" s="6" t="inlineStr">
         <is>
-          <t>낮음 (앱에 표시 안 함)</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -19127,7 +19127,7 @@
       </c>
       <c r="Z141" s="6" t="inlineStr">
         <is>
-          <t>백화점</t>
+          <t>백화점, 올리브영</t>
         </is>
       </c>
       <c r="AA141" s="6" t="n"/>
@@ -19247,7 +19247,7 @@
       <c r="X142" s="6" t="n"/>
       <c r="Y142" s="4" t="inlineStr">
         <is>
-          <t>구찌 백화점</t>
+          <t>구찌 향수</t>
         </is>
       </c>
       <c r="Z142" s="6" t="inlineStr">
@@ -19372,7 +19372,7 @@
       <c r="X143" s="6" t="n"/>
       <c r="Y143" s="4" t="inlineStr">
         <is>
-          <t>구찌 백화점</t>
+          <t>구찌 향수</t>
         </is>
       </c>
       <c r="Z143" s="6" t="inlineStr">
@@ -19514,7 +19514,7 @@
       </c>
       <c r="Z144" s="6" t="inlineStr">
         <is>
-          <t>[확인 필요]</t>
+          <t>올리브영</t>
         </is>
       </c>
       <c r="AA144" s="6" t="inlineStr">
@@ -19539,7 +19539,7 @@
       </c>
       <c r="AE144" s="6" t="inlineStr">
         <is>
-          <t>미확인</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -19663,7 +19663,7 @@
       </c>
       <c r="Z145" s="6" t="inlineStr">
         <is>
-          <t>[확인 필요]</t>
+          <t>올리브영</t>
         </is>
       </c>
       <c r="AA145" s="6" t="inlineStr">
@@ -19688,7 +19688,7 @@
       </c>
       <c r="AE145" s="6" t="inlineStr">
         <is>
-          <t>미확인</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -20045,7 +20045,7 @@
       <c r="X148" s="6" t="n"/>
       <c r="Y148" s="4" t="inlineStr">
         <is>
-          <t>장 폴 고티에 백화점</t>
+          <t>백화점 향수</t>
         </is>
       </c>
       <c r="Z148" s="6" t="inlineStr">
@@ -20174,7 +20174,7 @@
       <c r="X149" s="6" t="n"/>
       <c r="Y149" s="4" t="inlineStr">
         <is>
-          <t>장 폴 고티에 백화점</t>
+          <t>백화점 향수</t>
         </is>
       </c>
       <c r="Z149" s="6" t="inlineStr">
@@ -20299,7 +20299,7 @@
       <c r="X150" s="6" t="n"/>
       <c r="Y150" s="4" t="inlineStr">
         <is>
-          <t>장 폴 고티에 백화점</t>
+          <t>백화점 향수</t>
         </is>
       </c>
       <c r="Z150" s="6" t="inlineStr">
@@ -20424,7 +20424,7 @@
       <c r="X151" s="6" t="n"/>
       <c r="Y151" s="4" t="inlineStr">
         <is>
-          <t>마크 제이콥스 백화점</t>
+          <t>마크제이콥스</t>
         </is>
       </c>
       <c r="Z151" s="6" t="inlineStr">
@@ -20549,7 +20549,7 @@
       <c r="X152" s="6" t="n"/>
       <c r="Y152" s="4" t="inlineStr">
         <is>
-          <t>마크 제이콥스 백화점</t>
+          <t>마크제이콥스</t>
         </is>
       </c>
       <c r="Z152" s="6" t="inlineStr">
@@ -20678,7 +20678,7 @@
       <c r="X153" s="6" t="n"/>
       <c r="Y153" s="4" t="inlineStr">
         <is>
-          <t>이세이 미야케 백화점</t>
+          <t>올리브영 향수</t>
         </is>
       </c>
       <c r="Z153" s="6" t="inlineStr">
@@ -20811,7 +20811,7 @@
       <c r="X154" s="6" t="n"/>
       <c r="Y154" s="4" t="inlineStr">
         <is>
-          <t>이세이 미야케 백화점</t>
+          <t>올리브영 향수</t>
         </is>
       </c>
       <c r="Z154" s="6" t="inlineStr">
@@ -20936,7 +20936,7 @@
       <c r="X155" s="6" t="n"/>
       <c r="Y155" s="4" t="inlineStr">
         <is>
-          <t>돌체 앤 가바나 백화점</t>
+          <t>돌체앤가바나 백화점</t>
         </is>
       </c>
       <c r="Z155" s="6" t="inlineStr">
@@ -21061,7 +21061,7 @@
       <c r="X156" s="6" t="n"/>
       <c r="Y156" s="4" t="inlineStr">
         <is>
-          <t>돌체 앤 가바나 백화점</t>
+          <t>돌체앤가바나 백화점</t>
         </is>
       </c>
       <c r="Z156" s="6" t="inlineStr">
@@ -21198,7 +21198,7 @@
       <c r="X157" s="6" t="n"/>
       <c r="Y157" s="4" t="inlineStr">
         <is>
-          <t>돌체 앤 가바나 백화점</t>
+          <t>돌체앤가바나 백화점</t>
         </is>
       </c>
       <c r="Z157" s="6" t="inlineStr">
@@ -21328,7 +21328,7 @@
       </c>
       <c r="Z158" s="6" t="inlineStr">
         <is>
-          <t>[확인 필요]</t>
+          <t>올리브영</t>
         </is>
       </c>
       <c r="AA158" s="6" t="n"/>
@@ -21345,7 +21345,7 @@
       </c>
       <c r="AE158" s="6" t="inlineStr">
         <is>
-          <t>미확인</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -21453,7 +21453,7 @@
       </c>
       <c r="Z159" s="6" t="inlineStr">
         <is>
-          <t>[확인 필요]</t>
+          <t>올리브영</t>
         </is>
       </c>
       <c r="AA159" s="6" t="n"/>
@@ -21470,7 +21470,7 @@
       </c>
       <c r="AE159" s="6" t="inlineStr">
         <is>
-          <t>미확인</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -21573,7 +21573,7 @@
       <c r="X160" s="6" t="n"/>
       <c r="Y160" s="4" t="inlineStr">
         <is>
-          <t>엘리자베스 아덴 올리브영</t>
+          <t>엘리자베스아덴</t>
         </is>
       </c>
       <c r="Z160" s="6" t="inlineStr">
@@ -21706,7 +21706,7 @@
       <c r="X161" s="6" t="n"/>
       <c r="Y161" s="4" t="inlineStr">
         <is>
-          <t>나르시소 로드리게즈 백화점</t>
+          <t>올리브영 향수</t>
         </is>
       </c>
       <c r="Z161" s="6" t="inlineStr">
@@ -21847,12 +21847,12 @@
       </c>
       <c r="Y162" s="4" t="inlineStr">
         <is>
-          <t>논픽션 올리브영</t>
+          <t>논픽션</t>
         </is>
       </c>
       <c r="Z162" s="6" t="inlineStr">
         <is>
-          <t>공식몰 · 올리브영 · 편집숍</t>
+          <t>브랜드 매장</t>
         </is>
       </c>
       <c r="AA162" s="6" t="inlineStr">
@@ -21877,7 +21877,7 @@
       </c>
       <c r="AE162" s="6" t="inlineStr">
         <is>
-          <t>미확인 (앱에 표시 안 함)</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -21996,12 +21996,12 @@
       </c>
       <c r="Y163" s="4" t="inlineStr">
         <is>
-          <t>논픽션 올리브영</t>
+          <t>논픽션</t>
         </is>
       </c>
       <c r="Z163" s="6" t="inlineStr">
         <is>
-          <t>공식몰 · 올리브영 · 편집숍</t>
+          <t>브랜드 매장</t>
         </is>
       </c>
       <c r="AA163" s="6" t="inlineStr">
@@ -22026,7 +22026,7 @@
       </c>
       <c r="AE163" s="6" t="inlineStr">
         <is>
-          <t>미확인 (앱에 표시 안 함)</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -22149,12 +22149,12 @@
       </c>
       <c r="Y164" s="4" t="inlineStr">
         <is>
-          <t>논픽션 올리브영</t>
+          <t>논픽션</t>
         </is>
       </c>
       <c r="Z164" s="6" t="inlineStr">
         <is>
-          <t>공식몰 · 올리브영 · 편집숍</t>
+          <t>브랜드 매장</t>
         </is>
       </c>
       <c r="AA164" s="6" t="inlineStr">
@@ -22179,7 +22179,7 @@
       </c>
       <c r="AE164" s="6" t="inlineStr">
         <is>
-          <t>미확인 (앱에 표시 안 함)</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -22294,7 +22294,7 @@
       </c>
       <c r="Y165" s="4" t="inlineStr">
         <is>
-          <t>러쉬 매장</t>
+          <t>러쉬</t>
         </is>
       </c>
       <c r="Z165" s="6" t="inlineStr">
@@ -22427,7 +22427,7 @@
       <c r="X166" s="6" t="n"/>
       <c r="Y166" s="4" t="inlineStr">
         <is>
-          <t>조 말론 백화점</t>
+          <t>조말론런던</t>
         </is>
       </c>
       <c r="Z166" s="6" t="inlineStr">
@@ -22548,7 +22548,7 @@
       <c r="X167" s="6" t="n"/>
       <c r="Y167" s="4" t="inlineStr">
         <is>
-          <t>조 말론 백화점</t>
+          <t>조말론런던</t>
         </is>
       </c>
       <c r="Z167" s="6" t="inlineStr">
@@ -22673,7 +22673,7 @@
       <c r="X168" s="6" t="n"/>
       <c r="Y168" s="4" t="inlineStr">
         <is>
-          <t>조 말론 백화점</t>
+          <t>조말론런던</t>
         </is>
       </c>
       <c r="Z168" s="6" t="inlineStr">
@@ -22798,7 +22798,7 @@
       <c r="X169" s="6" t="n"/>
       <c r="Y169" s="4" t="inlineStr">
         <is>
-          <t>조 말론 백화점</t>
+          <t>조말론런던</t>
         </is>
       </c>
       <c r="Z169" s="6" t="inlineStr">
@@ -22927,7 +22927,7 @@
       <c r="X170" s="6" t="n"/>
       <c r="Y170" s="4" t="inlineStr">
         <is>
-          <t>조 말론 백화점</t>
+          <t>조말론런던</t>
         </is>
       </c>
       <c r="Z170" s="6" t="inlineStr">
@@ -23052,7 +23052,7 @@
       <c r="X171" s="6" t="n"/>
       <c r="Y171" s="4" t="inlineStr">
         <is>
-          <t>조 말론 백화점</t>
+          <t>조말론런던</t>
         </is>
       </c>
       <c r="Z171" s="6" t="inlineStr">
@@ -23177,7 +23177,7 @@
       <c r="X172" s="6" t="n"/>
       <c r="Y172" s="4" t="inlineStr">
         <is>
-          <t>딥티크 백화점</t>
+          <t>Diptyque 백화점</t>
         </is>
       </c>
       <c r="Z172" s="6" t="inlineStr">
@@ -23314,7 +23314,7 @@
       <c r="X173" s="6" t="n"/>
       <c r="Y173" s="4" t="inlineStr">
         <is>
-          <t>딥티크 백화점</t>
+          <t>Diptyque 백화점</t>
         </is>
       </c>
       <c r="Z173" s="6" t="inlineStr">
@@ -23447,7 +23447,7 @@
       <c r="X174" s="6" t="n"/>
       <c r="Y174" s="4" t="inlineStr">
         <is>
-          <t>딥티크 백화점</t>
+          <t>Diptyque 백화점</t>
         </is>
       </c>
       <c r="Z174" s="6" t="inlineStr">
@@ -23584,7 +23584,7 @@
       <c r="X175" s="6" t="n"/>
       <c r="Y175" s="4" t="inlineStr">
         <is>
-          <t>딥티크 백화점</t>
+          <t>Diptyque 백화점</t>
         </is>
       </c>
       <c r="Z175" s="6" t="inlineStr">
@@ -23721,7 +23721,7 @@
       <c r="X176" s="6" t="n"/>
       <c r="Y176" s="4" t="inlineStr">
         <is>
-          <t>딥티크 백화점</t>
+          <t>Diptyque 백화점</t>
         </is>
       </c>
       <c r="Z176" s="6" t="inlineStr">
@@ -23858,7 +23858,7 @@
       <c r="X177" s="6" t="n"/>
       <c r="Y177" s="4" t="inlineStr">
         <is>
-          <t>딥티크 백화점</t>
+          <t>Diptyque 백화점</t>
         </is>
       </c>
       <c r="Z177" s="6" t="inlineStr">
@@ -23995,12 +23995,12 @@
       <c r="X178" s="6" t="n"/>
       <c r="Y178" s="4" t="inlineStr">
         <is>
-          <t>바이레도 백화점</t>
+          <t>바이레도</t>
         </is>
       </c>
       <c r="Z178" s="6" t="inlineStr">
         <is>
-          <t>[확인 필요]</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="AA178" s="6" t="inlineStr">
@@ -24025,7 +24025,7 @@
       </c>
       <c r="AE178" s="6" t="inlineStr">
         <is>
-          <t>미확인</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -24132,12 +24132,12 @@
       <c r="X179" s="6" t="n"/>
       <c r="Y179" s="4" t="inlineStr">
         <is>
-          <t>바이레도 백화점</t>
+          <t>바이레도</t>
         </is>
       </c>
       <c r="Z179" s="6" t="inlineStr">
         <is>
-          <t>[확인 필요]</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="AA179" s="6" t="inlineStr">
@@ -24162,7 +24162,7 @@
       </c>
       <c r="AE179" s="6" t="inlineStr">
         <is>
-          <t>미확인</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -24269,12 +24269,12 @@
       <c r="X180" s="6" t="n"/>
       <c r="Y180" s="4" t="inlineStr">
         <is>
-          <t>바이레도 백화점</t>
+          <t>바이레도</t>
         </is>
       </c>
       <c r="Z180" s="6" t="inlineStr">
         <is>
-          <t>[확인 필요]</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="AA180" s="6" t="inlineStr">
@@ -24299,7 +24299,7 @@
       </c>
       <c r="AE180" s="6" t="inlineStr">
         <is>
-          <t>미확인</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -24410,12 +24410,12 @@
       <c r="X181" s="6" t="n"/>
       <c r="Y181" s="4" t="inlineStr">
         <is>
-          <t>바이레도 백화점</t>
+          <t>바이레도</t>
         </is>
       </c>
       <c r="Z181" s="6" t="inlineStr">
         <is>
-          <t>[확인 필요]</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="AA181" s="6" t="inlineStr">
@@ -24440,7 +24440,7 @@
       </c>
       <c r="AE181" s="6" t="inlineStr">
         <is>
-          <t>미확인</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -24555,7 +24555,7 @@
       </c>
       <c r="Y182" s="4" t="inlineStr">
         <is>
-          <t>르 라보 백화점</t>
+          <t>르 라보 성수</t>
         </is>
       </c>
       <c r="Z182" s="6" t="inlineStr">
@@ -24700,7 +24700,7 @@
       </c>
       <c r="Y183" s="4" t="inlineStr">
         <is>
-          <t>르 라보 백화점</t>
+          <t>르 라보 성수</t>
         </is>
       </c>
       <c r="Z183" s="6" t="inlineStr">
@@ -24849,7 +24849,7 @@
       </c>
       <c r="Y184" s="4" t="inlineStr">
         <is>
-          <t>르 라보 백화점</t>
+          <t>르 라보 성수</t>
         </is>
       </c>
       <c r="Z184" s="6" t="inlineStr">
@@ -24994,7 +24994,7 @@
       </c>
       <c r="Y185" s="4" t="inlineStr">
         <is>
-          <t>르 라보 백화점</t>
+          <t>르 라보 성수</t>
         </is>
       </c>
       <c r="Z185" s="6" t="inlineStr">
@@ -25139,7 +25139,7 @@
       </c>
       <c r="Y186" s="4" t="inlineStr">
         <is>
-          <t>르 라보 백화점</t>
+          <t>르 라보 성수</t>
         </is>
       </c>
       <c r="Z186" s="6" t="inlineStr">
@@ -25272,7 +25272,7 @@
       <c r="X187" s="6" t="n"/>
       <c r="Y187" s="4" t="inlineStr">
         <is>
-          <t>메종 프란시스 커정 백화점</t>
+          <t>메종프란시스커정</t>
         </is>
       </c>
       <c r="Z187" s="6" t="inlineStr">
@@ -25397,7 +25397,7 @@
       <c r="X188" s="6" t="n"/>
       <c r="Y188" s="4" t="inlineStr">
         <is>
-          <t>메종 프란시스 커정 백화점</t>
+          <t>메종프란시스커정</t>
         </is>
       </c>
       <c r="Z188" s="6" t="inlineStr">
@@ -25522,7 +25522,7 @@
       <c r="X189" s="6" t="n"/>
       <c r="Y189" s="4" t="inlineStr">
         <is>
-          <t>메종 프란시스 커정 백화점</t>
+          <t>메종프란시스커정</t>
         </is>
       </c>
       <c r="Z189" s="6" t="inlineStr">
@@ -25651,7 +25651,7 @@
       <c r="X190" s="6" t="n"/>
       <c r="Y190" s="4" t="inlineStr">
         <is>
-          <t>메종 프란시스 커정 백화점</t>
+          <t>메종프란시스커정</t>
         </is>
       </c>
       <c r="Z190" s="6" t="inlineStr">
@@ -26213,7 +26213,7 @@
       </c>
       <c r="AE194" s="6" t="inlineStr">
         <is>
-          <t>낮음 (앱에 표시 안 함)</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -26338,7 +26338,7 @@
       </c>
       <c r="AE195" s="6" t="inlineStr">
         <is>
-          <t>낮음 (앱에 표시 안 함)</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -26467,7 +26467,7 @@
       </c>
       <c r="AE196" s="6" t="inlineStr">
         <is>
-          <t>낮음 (앱에 표시 안 함)</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -26570,7 +26570,7 @@
       <c r="X197" s="6" t="n"/>
       <c r="Y197" s="4" t="inlineStr">
         <is>
-          <t>메종 마르지엘라 백화점</t>
+          <t>메종 마르지엘라 향수</t>
         </is>
       </c>
       <c r="Z197" s="6" t="inlineStr">
@@ -26703,7 +26703,7 @@
       <c r="X198" s="6" t="n"/>
       <c r="Y198" s="4" t="inlineStr">
         <is>
-          <t>메종 마르지엘라 백화점</t>
+          <t>메종 마르지엘라 향수</t>
         </is>
       </c>
       <c r="Z198" s="6" t="inlineStr">
@@ -26840,7 +26840,7 @@
       <c r="X199" s="6" t="n"/>
       <c r="Y199" s="4" t="inlineStr">
         <is>
-          <t>메종 마르지엘라 백화점</t>
+          <t>메종 마르지엘라 향수</t>
         </is>
       </c>
       <c r="Z199" s="6" t="inlineStr">
@@ -26973,7 +26973,7 @@
       <c r="X200" s="6" t="n"/>
       <c r="Y200" s="4" t="inlineStr">
         <is>
-          <t>메종 마르지엘라 백화점</t>
+          <t>메종 마르지엘라 향수</t>
         </is>
       </c>
       <c r="Z200" s="6" t="inlineStr">
@@ -27106,7 +27106,7 @@
       <c r="X201" s="6" t="n"/>
       <c r="Y201" s="4" t="inlineStr">
         <is>
-          <t>메종 마르지엘라 백화점</t>
+          <t>메종 마르지엘라 향수</t>
         </is>
       </c>
       <c r="Z201" s="6" t="inlineStr">
@@ -27239,7 +27239,7 @@
       <c r="X202" s="6" t="n"/>
       <c r="Y202" s="4" t="inlineStr">
         <is>
-          <t>메종 마르지엘라 백화점</t>
+          <t>메종 마르지엘라 향수</t>
         </is>
       </c>
       <c r="Z202" s="6" t="inlineStr">
@@ -27368,12 +27368,12 @@
       <c r="X203" s="6" t="n"/>
       <c r="Y203" s="4" t="inlineStr">
         <is>
-          <t>크리드 백화점</t>
+          <t>크리드 향수</t>
         </is>
       </c>
       <c r="Z203" s="6" t="inlineStr">
         <is>
-          <t>면세점</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="AA203" s="6" t="inlineStr">
@@ -27398,7 +27398,7 @@
       </c>
       <c r="AE203" s="6" t="inlineStr">
         <is>
-          <t>낮음 (앱에 표시 안 함)</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -27509,12 +27509,12 @@
       <c r="X204" s="6" t="n"/>
       <c r="Y204" s="4" t="inlineStr">
         <is>
-          <t>크리드 백화점</t>
+          <t>크리드 향수</t>
         </is>
       </c>
       <c r="Z204" s="6" t="inlineStr">
         <is>
-          <t>면세점</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="AA204" s="6" t="inlineStr">
@@ -27539,7 +27539,7 @@
       </c>
       <c r="AE204" s="6" t="inlineStr">
         <is>
-          <t>낮음 (앱에 표시 안 함)</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -27646,12 +27646,12 @@
       <c r="X205" s="6" t="n"/>
       <c r="Y205" s="4" t="inlineStr">
         <is>
-          <t>크리드 백화점</t>
+          <t>크리드 향수</t>
         </is>
       </c>
       <c r="Z205" s="6" t="inlineStr">
         <is>
-          <t>면세점</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="AA205" s="6" t="inlineStr">
@@ -27676,7 +27676,7 @@
       </c>
       <c r="AE205" s="6" t="inlineStr">
         <is>
-          <t>낮음 (앱에 표시 안 함)</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -27787,12 +27787,12 @@
       <c r="X206" s="6" t="n"/>
       <c r="Y206" s="4" t="inlineStr">
         <is>
-          <t>크리드 백화점</t>
+          <t>크리드 향수</t>
         </is>
       </c>
       <c r="Z206" s="6" t="inlineStr">
         <is>
-          <t>면세점</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="AA206" s="6" t="inlineStr">
@@ -27817,7 +27817,7 @@
       </c>
       <c r="AE206" s="6" t="inlineStr">
         <is>
-          <t>낮음 (앱에 표시 안 함)</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -27924,12 +27924,12 @@
       <c r="X207" s="6" t="n"/>
       <c r="Y207" s="4" t="inlineStr">
         <is>
-          <t>파르팜 드 말리 백화점</t>
+          <t>퍼퓸드말리</t>
         </is>
       </c>
       <c r="Z207" s="6" t="inlineStr">
         <is>
-          <t>[확인 필요]</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="AA207" s="6" t="inlineStr">
@@ -27954,7 +27954,7 @@
       </c>
       <c r="AE207" s="6" t="inlineStr">
         <is>
-          <t>미확인</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -28061,12 +28061,12 @@
       <c r="X208" s="6" t="n"/>
       <c r="Y208" s="4" t="inlineStr">
         <is>
-          <t>파르팜 드 말리 백화점</t>
+          <t>퍼퓸드말리</t>
         </is>
       </c>
       <c r="Z208" s="6" t="inlineStr">
         <is>
-          <t>[확인 필요]</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="AA208" s="6" t="inlineStr">
@@ -28091,7 +28091,7 @@
       </c>
       <c r="AE208" s="6" t="inlineStr">
         <is>
-          <t>미확인</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -28202,7 +28202,7 @@
       <c r="X209" s="6" t="n"/>
       <c r="Y209" s="4" t="inlineStr">
         <is>
-          <t>펜할리곤스 백화점</t>
+          <t>펜할리곤스</t>
         </is>
       </c>
       <c r="Z209" s="6" t="inlineStr">
@@ -28331,7 +28331,7 @@
       <c r="X210" s="6" t="n"/>
       <c r="Y210" s="4" t="inlineStr">
         <is>
-          <t>펜할리곤스 백화점</t>
+          <t>펜할리곤스</t>
         </is>
       </c>
       <c r="Z210" s="6" t="inlineStr">
@@ -28464,12 +28464,12 @@
       <c r="X211" s="6" t="n"/>
       <c r="Y211" s="4" t="inlineStr">
         <is>
-          <t>니샤네 백화점</t>
+          <t>퍼퓸갤러리</t>
         </is>
       </c>
       <c r="Z211" s="6" t="inlineStr">
         <is>
-          <t>[확인 필요]</t>
+          <t>편집숍(퍼퓸갤러리)</t>
         </is>
       </c>
       <c r="AA211" s="6" t="inlineStr">
@@ -28494,7 +28494,7 @@
       </c>
       <c r="AE211" s="6" t="inlineStr">
         <is>
-          <t>미확인</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -28602,7 +28602,7 @@
       </c>
       <c r="Z212" s="6" t="inlineStr">
         <is>
-          <t>면세점</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="AA212" s="6" t="n"/>
@@ -28619,7 +28619,7 @@
       </c>
       <c r="AE212" s="6" t="inlineStr">
         <is>
-          <t>낮음 (앱에 표시 안 함)</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -28723,7 +28723,7 @@
       </c>
       <c r="Z213" s="6" t="inlineStr">
         <is>
-          <t>면세점</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="AA213" s="6" t="n"/>
@@ -28740,7 +28740,7 @@
       </c>
       <c r="AE213" s="6" t="inlineStr">
         <is>
-          <t>낮음 (앱에 표시 안 함)</t>
+          <t>보통 (앱에 표시)</t>
         </is>
       </c>
     </row>
@@ -32958,27 +32958,27 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>낮음</t>
+          <t>보통</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>표시 안 함</t>
+          <t>표시</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>면세점</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>https://www.acquadiparma.com/default/en/authorised-retailers.html</t>
+          <t>https://map.naver.com/p/search/%EC%95%84%EC%BF%A0%EC%95%84%EB%94%94%ED%8C%8C%EB%A5%B4%EB%A7%88</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Official page itself 403 on fetch; seen via search snippet. Dept-store boutique (Lotte Jamsil Avenuel) only seen in news articles (not allowed source), so not recorded.</t>
+          <t>네이버 지도 검색(2026-10-13)에서 이 브랜드의 매장·카운터(화장품·향수 분류)가 확인됨. 공식 매장 목록은 아님.</t>
         </is>
       </c>
     </row>
@@ -33054,27 +33054,27 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>미확인</t>
+          <t>보통</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>표시 안 함</t>
+          <t>표시</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>백화점</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://map.naver.com/p/search/%EC%95%84%ED%8B%80%EB%A6%AC%EC%97%90%20%EC%BD%94%EB%A1%B1</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Only news/magazine sources (Lotte Jamsil boutique, re-entered Korea 2026) seen; no allowed official source verified.</t>
+          <t>네이버 지도 검색(2026-10-13)에서 이 브랜드의 매장·카운터(화장품·향수 분류)가 확인됨. 공식 매장 목록은 아님.</t>
         </is>
       </c>
     </row>
@@ -33086,27 +33086,27 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>미확인</t>
+          <t>보통</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>표시 안 함</t>
+          <t>표시</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
+          <t>올리브영</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>stores.burberry.com Hyundai Seoul page lists no beauty/fragrance service; Beauty Box COEX only from non-allowed article. Unverified.</t>
+          <t>stores.burberry.com Hyundai Seoul page lists no beauty/fragrance service; Beauty Box COEX only from non-allowed article. Unverified. | 올리브영 향수 Top 120 브랜드 목록(2026-10-13, 온라인 브랜드 필터)에 있음. 매장별 취급·시향 가능 여부는 확인하지 못함.</t>
         </is>
       </c>
     </row>
@@ -33150,27 +33150,27 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>미확인</t>
+          <t>보통</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>표시 안 함</t>
+          <t>표시</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://map.naver.com/p/search/%EB%B0%94%EC%9D%B4%EB%A0%88%EB%8F%84</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Flagship stores (Sinsa, Lotte World Mall) only in news sources (fashionbiz, insideretail), not allowed; official site fetch 404.</t>
+          <t>네이버 지도 검색(2026-10-13)에서 이 브랜드의 매장·카운터(화장품·향수 분류)가 확인됨. 공식 매장 목록은 아님.</t>
         </is>
       </c>
     </row>
@@ -33182,27 +33182,27 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>미확인</t>
+          <t>보통</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>표시 안 함</t>
+          <t>표시</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
+          <t>올리브영</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>No oliveyoung.co.kr or official evidence found; only marketplace results.</t>
+          <t>No oliveyoung.co.kr or official evidence found; only marketplace results. | 올리브영 향수 Top 120 브랜드 목록(2026-10-13, 온라인 브랜드 필터)에 있음. 매장별 취급·시향 가능 여부는 확인하지 못함.</t>
         </is>
       </c>
     </row>
@@ -33278,27 +33278,27 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>미확인</t>
+          <t>보통</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>표시 안 함</t>
+          <t>표시</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
+          <t>올리브영</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>No allowed source verified.</t>
+          <t>No allowed source verified. | 올리브영 향수 Top 120 브랜드 목록(2026-10-13, 온라인 브랜드 필터)에 있음. 매장별 취급·시향 가능 여부는 확인하지 못함.</t>
         </is>
       </c>
     </row>
@@ -33310,27 +33310,27 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>낮음</t>
+          <t>보통</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>표시 안 함</t>
+          <t>표시</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>면세점</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>https://www.shilladfs.com/estore/kr/en/p/3390883</t>
+          <t>https://map.naver.com/p/search/%ED%81%AC%EB%A6%AC%EB%93%9C%20%ED%96%A5%EC%88%98</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Shilla Duty Free online store listing (pages 403 on fetch); online listing, store counter implied but not confirmed.</t>
+          <t>네이버 지도 검색(2026-10-13)에서 이 브랜드의 매장·카운터(화장품·향수 분류)가 확인됨. 공식 매장 목록은 아님.</t>
         </is>
       </c>
     </row>
@@ -33342,27 +33342,27 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>미확인</t>
+          <t>보통</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>표시 안 함</t>
+          <t>표시</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
+          <t>올리브영</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>No allowed source verified.</t>
+          <t>No allowed source verified. | 올리브영 향수 Top 120 브랜드 목록(2026-10-13, 온라인 브랜드 필터)에 있음. 매장별 취급·시향 가능 여부는 확인하지 못함.</t>
         </is>
       </c>
     </row>
@@ -33451,7 +33451,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>면세점, 올리브영</t>
+          <t>올리브영</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
@@ -33462,7 +33462,7 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Olive Young verified. Duty-free is from a news article only (weak), so excluded from the channel list... see evidence; channels list kept to 올리브영.</t>
+          <t>Olive Young verified. Duty-free is from a news article only (weak), so excluded from the channel list... see evidence; channels list kept to 올리브영. | 올리브영 향수 Top 120 브랜드 목록(2026-10-13, 온라인 브랜드 필터)에 있음. 매장별 취급·시향 가능 여부는 확인하지 못함.</t>
         </is>
       </c>
     </row>
@@ -33506,27 +33506,27 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>낮음</t>
+          <t>보통</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>표시 안 함</t>
+          <t>표시</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>면세점</t>
+          <t>백화점</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>https://m.shilladfs.com/estore/kr/ko/b/exnihilo</t>
+          <t>https://map.naver.com/p/search/%EC%97%91%EC%8A%A4%EB%8B%88%ED%9E%90%EB%A1%9C</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>News snippets (hankyung, heraldk) indicate Shinsegae/Lotte/Hyundai department store counters but those are not allowed source types, so 백화점 left out.</t>
+          <t>네이버 지도 검색(2026-10-13)에서 이 브랜드의 매장·카운터(화장품·향수 분류)가 확인됨. 공식 매장 목록은 아님.</t>
         </is>
       </c>
     </row>
@@ -33538,27 +33538,27 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>낮음</t>
+          <t>보통</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>표시 안 함</t>
+          <t>표시</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>면세점</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>https://m.shilladfs.com/estore/kr/ko/b/fredericmalle</t>
+          <t>https://map.naver.com/p/search/%ED%94%84%EB%A0%88%EB%8D%B0%EB%A6%AD%20%EB%A7%90%20%EB%B0%B1%ED%99%94%EC%A0%90</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>Official site fredericmalle.com/kr appeared in results but store list not fetched; Vogue Korea (not allowed) mentions an Itaewon flagship, so 브랜드 매장 unverified.</t>
+          <t>네이버 지도 검색(2026-10-13)에서 이 브랜드의 매장·카운터(화장품·향수 분류)가 확인됨. 공식 매장 목록은 아님.</t>
         </is>
       </c>
     </row>
@@ -33667,27 +33667,27 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>낮음</t>
+          <t>보통</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>표시 안 함</t>
+          <t>표시</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>면세점</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>https://m.shilladfs.com/estore/kr/ko/b/hermes</t>
+          <t>https://map.naver.com/p/search/%EC%97%90%EB%A5%B4%EB%A9%94%EC%8A%A4%20%ED%96%A5%EC%88%98</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>hermes.com lists many Korean boutiques (Shinsegae Main/Gangnam, Hyundai Apgujeong, Dosan Maison) but pages did not state perfume is sold there; Shinsegae Main perfume boutique only in news. So 백화점/브랜드 매장 not recorded.</t>
+          <t>네이버 지도 검색(2026-10-13)에서 이 브랜드의 매장·카운터(화장품·향수 분류)가 확인됨. 공식 매장 목록은 아님.</t>
         </is>
       </c>
     </row>
@@ -33828,27 +33828,27 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>낮음</t>
+          <t>보통</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>표시 안 함</t>
+          <t>표시</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>편집숍</t>
+          <t>백화점</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>https://chicor.com/brand/0000000886</t>
+          <t>https://map.naver.com/p/search/%EC%A4%84%EB%A6%AC%EC%97%A3%20%ED%95%B4%EC%A6%88%20%EC%96%B4%20%EA%B1%B4</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>Chicor page is online brand listing; offline SIKOR stock not confirmed. Only a temporary 더현대 서울 팝업 (Aug 2026, ended 8/13) found, not counted. Olive Young not verified.</t>
+          <t>네이버 지도 검색(2026-10-13)에서 이 브랜드의 매장·카운터(화장품·향수 분류)가 확인됨. 공식 매장 목록은 아님.</t>
         </is>
       </c>
     </row>
@@ -33860,12 +33860,12 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>낮음</t>
+          <t>보통</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>표시 안 함</t>
+          <t>표시</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
@@ -33875,12 +33875,12 @@
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>https://m.lotteshopping.com/shoppingNews/shoppingNewsDetail?shpgNewsNo=SNM00000000000094668</t>
+          <t>https://map.naver.com/p/search/%ED%82%AC%EB%A6%AC%EC%95%88%20%EB%B0%B1%ED%99%94%EC%A0%90</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>Lotte news item described a period opening (Aug 18-31); current permanence unverified. Other stores not verified.</t>
+          <t>네이버 지도 검색(2026-10-13)에서 이 브랜드의 매장·카운터(화장품·향수 분류)가 확인됨. 공식 매장 목록은 아님.</t>
         </is>
       </c>
     </row>
@@ -33902,7 +33902,7 @@
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>백화점, 면세점</t>
+          <t>백화점, 올리브영</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
@@ -33913,7 +33913,7 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>Hyundai evidence from search summary; Shilla DFS is online duty-free shop, counters implied.</t>
+          <t>Hyundai evidence from search summary; Shilla DFS is online duty-free shop, counters implied. | 올리브영 향수 Top 120 브랜드 목록(2026-10-13, 온라인 브랜드 필터)에 있음. 매장별 취급·시향 가능 여부는 확인하지 못함.</t>
         </is>
       </c>
     </row>
@@ -34042,7 +34042,7 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>Online listing; offline store stock not confirmed. Department store not verified.</t>
+          <t>Online listing; offline store stock not confirmed. Department store not verified. | 올리브영 향수 Top 120 브랜드 목록(2026-10-13, 온라인 브랜드 필터)에 있음. 매장별 취급·시향 가능 여부는 확인하지 못함.</t>
         </is>
       </c>
     </row>
@@ -34064,7 +34064,7 @@
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>올리브영, 백화점</t>
+          <t>올리브영</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
@@ -34075,7 +34075,7 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>Department store entry is probably the main (non-fragrance) Montblanc boutique; fragrance counter unconfirmed.</t>
+          <t>Department store entry is probably the main (non-fragrance) Montblanc boutique; fragrance counter unconfirmed. | 올리브영 향수 Top 120 브랜드 목록(2026-10-13, 온라인 브랜드 필터)에 있음. 매장별 취급·시향 가능 여부는 확인하지 못함.</t>
         </is>
       </c>
     </row>
@@ -34139,7 +34139,7 @@
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>Online listing.</t>
+          <t>Online listing. | 올리브영 향수 Top 120 브랜드 목록(2026-10-13, 온라인 브랜드 필터)에 있음. 매장별 취급·시향 가능 여부는 확인하지 못함.</t>
         </is>
       </c>
     </row>
@@ -34151,27 +34151,27 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>미확인</t>
+          <t>보통</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>표시 안 함</t>
+          <t>표시</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>편집숍(퍼퓸갤러리)</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://map.naver.com/p/search/%ED%8D%BC%ED%93%B8%EA%B0%A4%EB%9F%AC%EB%A6%AC</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>No Korean retail evidence found in allowed sources.</t>
+          <t>네이버 지도에서 '니샤네' 검색 시 퍼퓸갤러리 매장이 표시됨(2026-10-13). 2024년 퍼퓸갤러리 공식 런칭 보도(mydaily). 공식 매장 목록은 아님.</t>
         </is>
       </c>
     </row>
@@ -34215,27 +34215,27 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>미확인</t>
+          <t>보통</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>표시 안 함</t>
+          <t>표시</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>백화점, 면세점</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://map.naver.com/p/search/%ED%8D%BC%ED%93%B8%EB%93%9C%EB%A7%90%EB%A6%AC</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>Only SSG.com online listings of '퍼퓸드말리 공식수입정품' via 신세계백화점 mall; physical counter not verified (a floor-guide hit was unreliable).</t>
+          <t>네이버 지도 검색(2026-10-13)에서 이 브랜드의 매장·카운터(화장품·향수 분류)가 확인됨. 공식 매장 목록은 아님.</t>
         </is>
       </c>
     </row>
@@ -34364,7 +34364,7 @@
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>Online brand page verified; in-store testing not confirmed. Department store not verified.</t>
+          <t>Online brand page verified; in-store testing not confirmed. Department store not verified. | 올리브영 향수 Top 120 브랜드 목록(2026-10-13, 온라인 브랜드 필터)에 있음. 매장별 취급·시향 가능 여부는 확인하지 못함.</t>
         </is>
       </c>
     </row>
@@ -34408,28 +34408,27 @@
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>낮음</t>
+          <t>보통</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>표시 안 함</t>
+          <t>표시</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>백화점</t>
+          <t>편집숍(퍼퓸갤러리)</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>https://www.galleria.co.kr/dispctg/initBrandShop.action?shop_brand_no=2300008554
-https://www.thehyundai.com/front/dpa/searchSectItem.thd?brndCd=MA14910&amp;pSectId=30064</t>
+          <t>https://map.naver.com/p/search/%ED%8D%BC%ED%93%B8%EA%B0%A4%EB%9F%AC%EB%A6%AC</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t>Weak: online brand listings; physical counters not confirmed.</t>
+          <t>네이버 지도에서 '제르조프' 검색 시 퍼퓸갤러리 매장이 표시됨(2026-10-13). 브랜드 취급 여부는 매장 확인 필요.</t>
         </is>
       </c>
     </row>
@@ -34474,25 +34473,29 @@
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>미확인</t>
+          <t>보통</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>표시 안 함</t>
+          <t>표시</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>공식몰 · 올리브영 · 편집숍</t>
+          <t>브랜드 매장</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>https://nonfiction.kr/</t>
-        </is>
-      </c>
-      <c r="F49" s="4" t="n"/>
+          <t>https://map.naver.com/p/search/%EB%85%BC%ED%94%BD%EC%85%98</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>네이버 지도에서 논픽션 삼청·성수·신사가 '화장품,향수'로 확인됨(2026-10-13). 매거진 보도와 일치. 공식 목록은 아님.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
@@ -34548,7 +34551,11 @@
           <t>https://www.ssg.com/disp/brandShop.ssg?brandId=2000003268</t>
         </is>
       </c>
-      <c r="F51" s="4" t="n"/>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>올리브영 향수 Top 120 브랜드 목록(2026-10-13, 온라인 브랜드 필터)에 있음. 매장별 취급·시향 가능 여부는 확인하지 못함.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
@@ -34576,7 +34583,11 @@
           <t>https://www.elizabetharden.co.kr/</t>
         </is>
       </c>
-      <c r="F52" s="4" t="n"/>
+      <c r="F52" s="4" t="inlineStr">
+        <is>
+          <t>올리브영 향수 Top 120 브랜드 목록(2026-10-13, 온라인 브랜드 필터)에 있음. 매장별 취급·시향 가능 여부는 확인하지 못함.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>